<commit_message>
Fix borders and relocate defect color legend below Top 5 defect table
</commit_message>
<xml_diff>
--- a/Database/HFPA_Template.xlsx
+++ b/Database/HFPA_Template.xlsx
@@ -1054,7 +1054,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="42">
+  <borders count="43">
     <border>
       <left/>
       <right/>
@@ -1558,6 +1558,17 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1703,7 +1714,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="244">
+  <cellXfs count="257">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -2334,6 +2345,29 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="121" borderId="36" pivotButton="0" quotePrefix="0" xfId="6"/>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="35" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="6">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="40" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="44" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="120" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="43" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="45" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="47" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="49" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="121" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="50">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2754,7 +2788,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X64"/>
+  <dimension ref="A1:X65"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.81666666666667" defaultRowHeight="17.25"/>
   <cols>
     <col width="8.81666666666667" customWidth="1" style="1" min="1" max="1"/>
@@ -2784,7 +2818,11 @@
           <t>FTY</t>
         </is>
       </c>
-      <c r="B1" s="85" t="n"/>
+      <c r="B1" s="85" t="inlineStr">
+        <is>
+          <t>Total pair produced</t>
+        </is>
+      </c>
       <c r="C1" s="86" t="inlineStr">
         <is>
           <t>Jan</t>
@@ -2850,6 +2888,8 @@
           <t>From Dec, 2025 report, change the rule to calculate % by model: FTT DR% by model= DR qty by model/Total inspection qty of all model of that factory. Sort model qty from highest to lowest then take top5</t>
         </is>
       </c>
+      <c r="U1" s="80" t="n"/>
+      <c r="V1" s="80" t="n"/>
     </row>
     <row r="2" ht="19" customHeight="1">
       <c r="A2" s="88" t="inlineStr">
@@ -2890,6 +2930,8 @@
       <c r="L2" s="90" t="n"/>
       <c r="M2" s="90" t="n"/>
       <c r="N2" s="91" t="n"/>
+      <c r="U2" s="80" t="n"/>
+      <c r="V2" s="80" t="n"/>
     </row>
     <row r="3" ht="19" customHeight="1">
       <c r="A3" s="88" t="inlineStr">
@@ -2930,6 +2972,8 @@
       <c r="L3" s="90" t="n"/>
       <c r="M3" s="90" t="n"/>
       <c r="N3" s="91" t="n"/>
+      <c r="U3" s="80" t="n"/>
+      <c r="V3" s="80" t="n"/>
     </row>
     <row r="4" ht="19" customHeight="1">
       <c r="A4" s="88" t="inlineStr">
@@ -2970,6 +3014,8 @@
       <c r="L4" s="90" t="n"/>
       <c r="M4" s="90" t="n"/>
       <c r="N4" s="91" t="n"/>
+      <c r="U4" s="80" t="n"/>
+      <c r="V4" s="80" t="n"/>
     </row>
     <row r="5" ht="19" customHeight="1">
       <c r="A5" s="88" t="inlineStr">
@@ -3011,6 +3057,8 @@
       <c r="M5" s="90" t="n"/>
       <c r="N5" s="91" t="n"/>
       <c r="P5" s="17" t="n"/>
+      <c r="U5" s="80" t="n"/>
+      <c r="V5" s="80" t="n"/>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="92" t="inlineStr">
@@ -3071,6 +3119,8 @@
         <f>SUM(N2:N5)</f>
         <v/>
       </c>
+      <c r="U6" s="80" t="n"/>
+      <c r="V6" s="80" t="n"/>
     </row>
     <row r="7" ht="14" customHeight="1">
       <c r="A7" s="80" t="n"/>
@@ -3092,6 +3142,11 @@
       <c r="Q7" s="80" t="n"/>
       <c r="R7" s="80" t="n"/>
       <c r="S7" s="80" t="n"/>
+      <c r="T7" s="80" t="n"/>
+      <c r="U7" s="80" t="n"/>
+      <c r="V7" s="80" t="n"/>
+      <c r="W7" s="80" t="n"/>
+      <c r="X7" s="80" t="n"/>
     </row>
     <row r="8" ht="24" customHeight="1">
       <c r="A8" s="84" t="inlineStr">
@@ -3099,7 +3154,11 @@
           <t>FTY</t>
         </is>
       </c>
-      <c r="B8" s="85" t="n"/>
+      <c r="B8" s="85" t="inlineStr">
+        <is>
+          <t>Defect</t>
+        </is>
+      </c>
       <c r="C8" s="86" t="inlineStr">
         <is>
           <t>Jan</t>
@@ -3160,6 +3219,8 @@
           <t>Dec</t>
         </is>
       </c>
+      <c r="U8" s="80" t="n"/>
+      <c r="V8" s="80" t="n"/>
     </row>
     <row r="9" ht="19" customHeight="1">
       <c r="A9" s="88" t="inlineStr">
@@ -3200,6 +3261,8 @@
       <c r="L9" s="90" t="n"/>
       <c r="M9" s="90" t="n"/>
       <c r="N9" s="91" t="n"/>
+      <c r="U9" s="80" t="n"/>
+      <c r="V9" s="80" t="n"/>
     </row>
     <row r="10" ht="19" customHeight="1">
       <c r="A10" s="88" t="inlineStr">
@@ -3240,6 +3303,8 @@
       <c r="L10" s="90" t="n"/>
       <c r="M10" s="90" t="n"/>
       <c r="N10" s="91" t="n"/>
+      <c r="U10" s="80" t="n"/>
+      <c r="V10" s="80" t="n"/>
     </row>
     <row r="11" ht="19" customHeight="1">
       <c r="A11" s="88" t="inlineStr">
@@ -3280,6 +3345,8 @@
       <c r="L11" s="90" t="n"/>
       <c r="M11" s="90" t="n"/>
       <c r="N11" s="91" t="n"/>
+      <c r="U11" s="80" t="n"/>
+      <c r="V11" s="80" t="n"/>
     </row>
     <row r="12" ht="19" customHeight="1">
       <c r="A12" s="88" t="inlineStr">
@@ -3320,6 +3387,8 @@
       <c r="L12" s="90" t="n"/>
       <c r="M12" s="90" t="n"/>
       <c r="N12" s="91" t="n"/>
+      <c r="U12" s="80" t="n"/>
+      <c r="V12" s="80" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="92" t="inlineStr">
@@ -3380,6 +3449,8 @@
         <f>SUM(N9:N12)</f>
         <v/>
       </c>
+      <c r="U13" s="80" t="n"/>
+      <c r="V13" s="80" t="n"/>
     </row>
     <row r="14" ht="14" customHeight="1">
       <c r="A14" s="80" t="n"/>
@@ -3401,6 +3472,11 @@
       <c r="Q14" s="80" t="n"/>
       <c r="R14" s="80" t="n"/>
       <c r="S14" s="80" t="n"/>
+      <c r="T14" s="80" t="n"/>
+      <c r="U14" s="80" t="n"/>
+      <c r="V14" s="80" t="n"/>
+      <c r="W14" s="80" t="n"/>
+      <c r="X14" s="80" t="n"/>
     </row>
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="84" t="inlineStr">
@@ -3478,6 +3554,8 @@
       <c r="R15" s="17" t="n"/>
       <c r="S15" s="17" t="n"/>
       <c r="T15" s="17" t="n"/>
+      <c r="U15" s="80" t="n"/>
+      <c r="V15" s="80" t="n"/>
     </row>
     <row r="16" ht="19" customHeight="1">
       <c r="A16" s="88" t="inlineStr">
@@ -3491,54 +3569,56 @@
         </is>
       </c>
       <c r="C16" s="96">
-        <f>1-C9/C2</f>
+        <f>IF(C2&gt;0, 1-C9/C2, "")</f>
         <v/>
       </c>
       <c r="D16" s="96">
-        <f>1-D9/D2</f>
+        <f>IF(D2&gt;0, 1-D9/D2, "")</f>
         <v/>
       </c>
       <c r="E16" s="96">
-        <f>1-E9/E2</f>
+        <f>IF(E2&gt;0, 1-E9/E2, "")</f>
         <v/>
       </c>
       <c r="F16" s="96">
-        <f>1-F9/F2</f>
+        <f>IF(F2&gt;0, 1-F9/F2, "")</f>
         <v/>
       </c>
       <c r="G16" s="96">
-        <f>1-G9/G2</f>
+        <f>IF(G2&gt;0, 1-G9/G2, "")</f>
         <v/>
       </c>
       <c r="H16" s="96">
-        <f>1-H9/H2</f>
+        <f>IF(H2&gt;0, 1-H9/H2, "")</f>
         <v/>
       </c>
       <c r="I16" s="96">
-        <f>1-I9/I2</f>
+        <f>IF(I2&gt;0, 1-I9/I2, "")</f>
         <v/>
       </c>
       <c r="J16" s="96">
-        <f>1-J9/J2</f>
+        <f>IF(J2&gt;0, 1-J9/J2, "")</f>
         <v/>
       </c>
       <c r="K16" s="96">
-        <f>1-K9/K2</f>
+        <f>IF(K2&gt;0, 1-K9/K2, "")</f>
         <v/>
       </c>
       <c r="L16" s="96">
-        <f>1-L9/L2</f>
+        <f>IF(L2&gt;0, 1-L9/L2, "")</f>
         <v/>
       </c>
       <c r="M16" s="96">
-        <f>1-M9/M2</f>
+        <f>IF(M2&gt;0, 1-M9/M2, "")</f>
         <v/>
       </c>
       <c r="N16" s="97">
-        <f>1-N9/N2</f>
+        <f>IF(N2&gt;0, 1-N9/N2, "")</f>
         <v/>
       </c>
       <c r="P16" s="17" t="n"/>
+      <c r="U16" s="80" t="n"/>
+      <c r="V16" s="80" t="n"/>
     </row>
     <row r="17" ht="19" customHeight="1">
       <c r="A17" s="88" t="inlineStr">
@@ -3552,54 +3632,56 @@
         </is>
       </c>
       <c r="C17" s="96">
-        <f>1-C10/C3</f>
+        <f>IF(C3&gt;0, 1-C10/C3, "")</f>
         <v/>
       </c>
       <c r="D17" s="96">
-        <f>1-D10/D3</f>
+        <f>IF(D3&gt;0, 1-D10/D3, "")</f>
         <v/>
       </c>
       <c r="E17" s="96">
-        <f>1-E10/E3</f>
+        <f>IF(E3&gt;0, 1-E10/E3, "")</f>
         <v/>
       </c>
       <c r="F17" s="96">
-        <f>1-F10/F3</f>
+        <f>IF(F3&gt;0, 1-F10/F3, "")</f>
         <v/>
       </c>
       <c r="G17" s="96">
-        <f>1-G10/G3</f>
+        <f>IF(G3&gt;0, 1-G10/G3, "")</f>
         <v/>
       </c>
       <c r="H17" s="96">
-        <f>1-H10/H3</f>
+        <f>IF(H3&gt;0, 1-H10/H3, "")</f>
         <v/>
       </c>
       <c r="I17" s="96">
-        <f>1-I10/I3</f>
+        <f>IF(I3&gt;0, 1-I10/I3, "")</f>
         <v/>
       </c>
       <c r="J17" s="96">
-        <f>1-J10/J3</f>
+        <f>IF(J3&gt;0, 1-J10/J3, "")</f>
         <v/>
       </c>
       <c r="K17" s="96">
-        <f>1-K10/K3</f>
+        <f>IF(K3&gt;0, 1-K10/K3, "")</f>
         <v/>
       </c>
       <c r="L17" s="96">
-        <f>1-L10/L3</f>
+        <f>IF(L3&gt;0, 1-L10/L3, "")</f>
         <v/>
       </c>
       <c r="M17" s="96">
-        <f>1-M10/M3</f>
+        <f>IF(M3&gt;0, 1-M10/M3, "")</f>
         <v/>
       </c>
       <c r="N17" s="97">
-        <f>1-N10/N3</f>
+        <f>IF(N3&gt;0, 1-N10/N3, "")</f>
         <v/>
       </c>
       <c r="P17" s="17" t="n"/>
+      <c r="U17" s="80" t="n"/>
+      <c r="V17" s="80" t="n"/>
     </row>
     <row r="18" ht="19" customHeight="1">
       <c r="A18" s="88" t="inlineStr">
@@ -3613,54 +3695,56 @@
         </is>
       </c>
       <c r="C18" s="96">
-        <f>1-C11/C4</f>
+        <f>IF(C4&gt;0, 1-C11/C4, "")</f>
         <v/>
       </c>
       <c r="D18" s="96">
-        <f>1-D11/D4</f>
+        <f>IF(D4&gt;0, 1-D11/D4, "")</f>
         <v/>
       </c>
       <c r="E18" s="96">
-        <f>1-E11/E4</f>
+        <f>IF(E4&gt;0, 1-E11/E4, "")</f>
         <v/>
       </c>
       <c r="F18" s="96">
-        <f>1-F11/F4</f>
+        <f>IF(F4&gt;0, 1-F11/F4, "")</f>
         <v/>
       </c>
       <c r="G18" s="96">
-        <f>1-G11/G4</f>
+        <f>IF(G4&gt;0, 1-G11/G4, "")</f>
         <v/>
       </c>
       <c r="H18" s="96">
-        <f>1-H11/H4</f>
+        <f>IF(H4&gt;0, 1-H11/H4, "")</f>
         <v/>
       </c>
       <c r="I18" s="96">
-        <f>1-I11/I4</f>
+        <f>IF(I4&gt;0, 1-I11/I4, "")</f>
         <v/>
       </c>
       <c r="J18" s="96">
-        <f>1-J11/J4</f>
+        <f>IF(J4&gt;0, 1-J11/J4, "")</f>
         <v/>
       </c>
       <c r="K18" s="96">
-        <f>1-K11/K4</f>
+        <f>IF(K4&gt;0, 1-K11/K4, "")</f>
         <v/>
       </c>
       <c r="L18" s="96">
-        <f>1-L11/L4</f>
+        <f>IF(L4&gt;0, 1-L11/L4, "")</f>
         <v/>
       </c>
       <c r="M18" s="96">
-        <f>1-M11/M4</f>
+        <f>IF(M4&gt;0, 1-M11/M4, "")</f>
         <v/>
       </c>
       <c r="N18" s="97">
-        <f>1-N11/N4</f>
+        <f>IF(N4&gt;0, 1-N11/N4, "")</f>
         <v/>
       </c>
       <c r="P18" s="17" t="n"/>
+      <c r="U18" s="80" t="n"/>
+      <c r="V18" s="80" t="n"/>
     </row>
     <row r="19" ht="19" customHeight="1">
       <c r="A19" s="88" t="inlineStr">
@@ -3674,54 +3758,56 @@
         </is>
       </c>
       <c r="C19" s="96">
-        <f>1-C12/C5</f>
+        <f>IF(C5&gt;0, 1-C12/C5, "")</f>
         <v/>
       </c>
       <c r="D19" s="96">
-        <f>1-D12/D5</f>
+        <f>IF(D5&gt;0, 1-D12/D5, "")</f>
         <v/>
       </c>
       <c r="E19" s="96">
-        <f>1-E12/E5</f>
+        <f>IF(E5&gt;0, 1-E12/E5, "")</f>
         <v/>
       </c>
       <c r="F19" s="96">
-        <f>1-F12/F5</f>
+        <f>IF(F5&gt;0, 1-F12/F5, "")</f>
         <v/>
       </c>
       <c r="G19" s="96">
-        <f>1-G12/G5</f>
+        <f>IF(G5&gt;0, 1-G12/G5, "")</f>
         <v/>
       </c>
       <c r="H19" s="96">
-        <f>1-H12/H5</f>
+        <f>IF(H5&gt;0, 1-H12/H5, "")</f>
         <v/>
       </c>
       <c r="I19" s="96">
-        <f>1-I12/I5</f>
+        <f>IF(I5&gt;0, 1-I12/I5, "")</f>
         <v/>
       </c>
       <c r="J19" s="96">
-        <f>1-J12/J5</f>
+        <f>IF(J5&gt;0, 1-J12/J5, "")</f>
         <v/>
       </c>
       <c r="K19" s="96">
-        <f>1-K12/K5</f>
+        <f>IF(K5&gt;0, 1-K12/K5, "")</f>
         <v/>
       </c>
       <c r="L19" s="96">
-        <f>1-L12/L5</f>
+        <f>IF(L5&gt;0, 1-L12/L5, "")</f>
         <v/>
       </c>
       <c r="M19" s="96">
-        <f>1-M12/M5</f>
+        <f>IF(M5&gt;0, 1-M12/M5, "")</f>
         <v/>
       </c>
       <c r="N19" s="97">
-        <f>1-N12/N5</f>
+        <f>IF(N5&gt;0, 1-N12/N5, "")</f>
         <v/>
       </c>
       <c r="P19" s="17" t="n"/>
+      <c r="U19" s="80" t="n"/>
+      <c r="V19" s="80" t="n"/>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="92" t="inlineStr">
@@ -3740,15 +3826,15 @@
       <c r="F20" s="98" t="n"/>
       <c r="G20" s="98" t="n"/>
       <c r="H20" s="100">
-        <f>1-H13/H6</f>
+        <f>IF(H6&gt;0, 1-H13/H6, "")</f>
         <v/>
       </c>
       <c r="I20" s="100">
-        <f>1-I13/I6</f>
+        <f>IF(I6&gt;0, 1-I13/I6, "")</f>
         <v/>
       </c>
       <c r="J20" s="100">
-        <f>1-J13/J6</f>
+        <f>IF(J6&gt;0, 1-J13/J6, "")</f>
         <v/>
       </c>
       <c r="K20" s="98" t="n"/>
@@ -3756,8 +3842,10 @@
       <c r="M20" s="98" t="n"/>
       <c r="N20" s="101" t="n"/>
       <c r="Q20" s="32" t="n"/>
-    </row>
-    <row r="21" ht="20" customHeight="1">
+      <c r="U20" s="80" t="n"/>
+      <c r="V20" s="80" t="n"/>
+    </row>
+    <row r="21" ht="24" customHeight="1">
       <c r="A21" s="80" t="n"/>
       <c r="B21" s="102" t="inlineStr">
         <is>
@@ -3831,21 +3919,17 @@
           <t>Components inconsistent</t>
         </is>
       </c>
-      <c r="R21" s="230" t="inlineStr">
+      <c r="R21" s="107" t="inlineStr">
         <is>
           <t>Midsole/Outsole to upper bond gap</t>
         </is>
       </c>
       <c r="S21" s="80" t="n"/>
       <c r="T21" s="80" t="n"/>
-      <c r="U21" s="126" t="inlineStr">
-        <is>
-          <t>Site VH</t>
-        </is>
-      </c>
-      <c r="V21" s="127" t="n"/>
-    </row>
-    <row r="22" ht="18" customHeight="1">
+      <c r="U21" s="244" t="n"/>
+      <c r="V21" s="80" t="n"/>
+    </row>
+    <row r="22" ht="19" customHeight="1">
       <c r="A22" s="80" t="n"/>
       <c r="B22" s="80" t="n"/>
       <c r="C22" s="108" t="inlineStr">
@@ -3892,18 +3976,14 @@
         <v>0.097844</v>
       </c>
       <c r="Q22" s="96" t="n"/>
-      <c r="R22" s="231" t="n"/>
+      <c r="R22" s="97" t="n"/>
       <c r="S22" s="83" t="n"/>
       <c r="T22" s="83" t="n"/>
-      <c r="U22" s="128" t="n"/>
-      <c r="V22" s="129" t="inlineStr">
-        <is>
-          <t>Cleanness</t>
-        </is>
-      </c>
+      <c r="U22" s="83" t="n"/>
+      <c r="V22" s="241" t="n"/>
       <c r="W22" s="24" t="n"/>
     </row>
-    <row r="23" ht="18" customHeight="1">
+    <row r="23" ht="19" customHeight="1">
       <c r="A23" s="80" t="n"/>
       <c r="B23" s="80" t="n"/>
       <c r="C23" s="113" t="n"/>
@@ -3942,18 +4022,14 @@
         <v>0.154912</v>
       </c>
       <c r="Q23" s="96" t="n"/>
-      <c r="R23" s="231" t="n"/>
+      <c r="R23" s="97" t="n"/>
       <c r="S23" s="83" t="n"/>
       <c r="T23" s="83" t="n"/>
-      <c r="U23" s="130" t="n"/>
-      <c r="V23" s="129" t="inlineStr">
-        <is>
-          <t>Over cement</t>
-        </is>
-      </c>
+      <c r="U23" s="83" t="n"/>
+      <c r="V23" s="241" t="n"/>
       <c r="W23" s="24" t="n"/>
     </row>
-    <row r="24" ht="18" customHeight="1">
+    <row r="24" ht="19" customHeight="1">
       <c r="A24" s="80" t="n"/>
       <c r="B24" s="80" t="n"/>
       <c r="C24" s="113" t="n"/>
@@ -3992,18 +4068,14 @@
       <c r="Q24" s="96" t="n">
         <v>0.126007</v>
       </c>
-      <c r="R24" s="231" t="n"/>
+      <c r="R24" s="97" t="n"/>
       <c r="S24" s="83" t="n"/>
       <c r="T24" s="83" t="n"/>
-      <c r="U24" s="132" t="n"/>
-      <c r="V24" s="129" t="inlineStr">
-        <is>
-          <t>Rocking</t>
-        </is>
-      </c>
+      <c r="U24" s="83" t="n"/>
+      <c r="V24" s="241" t="n"/>
       <c r="W24" s="24" t="n"/>
     </row>
-    <row r="25" ht="18" customHeight="1">
+    <row r="25" ht="19" customHeight="1">
       <c r="A25" s="80" t="n"/>
       <c r="B25" s="80" t="n"/>
       <c r="C25" s="113" t="n"/>
@@ -4042,18 +4114,14 @@
       </c>
       <c r="P25" s="96" t="n"/>
       <c r="Q25" s="96" t="n"/>
-      <c r="R25" s="231" t="n"/>
+      <c r="R25" s="97" t="n"/>
       <c r="S25" s="83" t="n"/>
       <c r="T25" s="83" t="n"/>
-      <c r="U25" s="136" t="n"/>
-      <c r="V25" s="129" t="inlineStr">
-        <is>
-          <t>Thread end</t>
-        </is>
-      </c>
+      <c r="U25" s="83" t="n"/>
+      <c r="V25" s="241" t="n"/>
       <c r="W25" s="24" t="n"/>
     </row>
-    <row r="26" ht="18" customHeight="1">
+    <row r="26" ht="19" customHeight="1">
       <c r="A26" s="80" t="n"/>
       <c r="B26" s="80" t="n"/>
       <c r="C26" s="115" t="n"/>
@@ -4090,20 +4158,16 @@
       </c>
       <c r="P26" s="119" t="n"/>
       <c r="Q26" s="119" t="n"/>
-      <c r="R26" s="231" t="n">
+      <c r="R26" s="120" t="n">
         <v>0.125621</v>
       </c>
       <c r="S26" s="83" t="n"/>
       <c r="T26" s="83" t="n"/>
-      <c r="U26" s="131" t="n"/>
-      <c r="V26" s="129" t="inlineStr">
-        <is>
-          <t>Components inconsistent</t>
-        </is>
-      </c>
+      <c r="U26" s="83" t="n"/>
+      <c r="V26" s="241" t="n"/>
       <c r="W26" s="24" t="n"/>
     </row>
-    <row r="27" ht="20" customHeight="1">
+    <row r="27" ht="24" customHeight="1">
       <c r="A27" s="80" t="n"/>
       <c r="B27" s="80" t="n"/>
       <c r="C27" s="84" t="inlineStr">
@@ -4172,14 +4236,10 @@
       <c r="R27" s="80" t="n"/>
       <c r="S27" s="80" t="n"/>
       <c r="T27" s="80" t="n"/>
-      <c r="U27" s="126" t="inlineStr">
-        <is>
-          <t>Site VH2</t>
-        </is>
-      </c>
-      <c r="V27" s="127" t="n"/>
-    </row>
-    <row r="28" ht="18" customHeight="1">
+      <c r="U27" s="244" t="n"/>
+      <c r="V27" s="80" t="n"/>
+    </row>
+    <row r="28" ht="19" customHeight="1">
       <c r="A28" s="80" t="n"/>
       <c r="B28" s="80" t="n"/>
       <c r="C28" s="108" t="inlineStr">
@@ -4229,14 +4289,10 @@
       <c r="R28" s="80" t="n"/>
       <c r="S28" s="80" t="n"/>
       <c r="T28" s="80" t="n"/>
-      <c r="U28" s="134" t="n"/>
-      <c r="V28" s="135" t="inlineStr">
-        <is>
-          <t>Cleanness</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="18" customHeight="1">
+      <c r="U28" s="80" t="n"/>
+      <c r="V28" s="245" t="n"/>
+    </row>
+    <row r="29" ht="19" customHeight="1">
       <c r="A29" s="80" t="n"/>
       <c r="B29" s="80" t="n"/>
       <c r="C29" s="113" t="n"/>
@@ -4278,15 +4334,11 @@
       <c r="R29" s="83" t="n"/>
       <c r="S29" s="83" t="n"/>
       <c r="T29" s="83" t="n"/>
-      <c r="U29" s="136" t="n"/>
-      <c r="V29" s="129" t="inlineStr">
-        <is>
-          <t>Thread end</t>
-        </is>
-      </c>
+      <c r="U29" s="83" t="n"/>
+      <c r="V29" s="241" t="n"/>
       <c r="W29" s="24" t="n"/>
     </row>
-    <row r="30" ht="18" customHeight="1">
+    <row r="30" ht="19" customHeight="1">
       <c r="A30" s="80" t="n"/>
       <c r="B30" s="80" t="n"/>
       <c r="C30" s="113" t="n"/>
@@ -4328,15 +4380,11 @@
       <c r="R30" s="83" t="n"/>
       <c r="S30" s="83" t="n"/>
       <c r="T30" s="83" t="n"/>
-      <c r="U30" s="130" t="n"/>
-      <c r="V30" s="129" t="inlineStr">
-        <is>
-          <t>Over cement</t>
-        </is>
-      </c>
+      <c r="U30" s="83" t="n"/>
+      <c r="V30" s="241" t="n"/>
       <c r="W30" s="24" t="n"/>
     </row>
-    <row r="31" ht="18" customHeight="1">
+    <row r="31" ht="19" customHeight="1">
       <c r="A31" s="80" t="n"/>
       <c r="B31" s="80" t="n"/>
       <c r="C31" s="113" t="n"/>
@@ -4378,15 +4426,11 @@
       <c r="R31" s="83" t="n"/>
       <c r="S31" s="83" t="n"/>
       <c r="T31" s="83" t="n"/>
-      <c r="U31" s="240" t="n"/>
-      <c r="V31" s="129" t="inlineStr">
-        <is>
-          <t>Airbag quality/stain</t>
-        </is>
-      </c>
+      <c r="U31" s="83" t="n"/>
+      <c r="V31" s="241" t="n"/>
       <c r="W31" s="24" t="n"/>
     </row>
-    <row r="32" ht="18" customHeight="1">
+    <row r="32" ht="19" customHeight="1">
       <c r="A32" s="80" t="n"/>
       <c r="B32" s="80" t="n"/>
       <c r="C32" s="115" t="n"/>
@@ -4428,15 +4472,11 @@
       <c r="R32" s="83" t="n"/>
       <c r="S32" s="83" t="n"/>
       <c r="T32" s="83" t="n"/>
-      <c r="U32" s="133" t="n"/>
-      <c r="V32" s="129" t="inlineStr">
-        <is>
-          <t>Midsole/Outsole to upper bond gap</t>
-        </is>
-      </c>
+      <c r="U32" s="83" t="n"/>
+      <c r="V32" s="241" t="n"/>
       <c r="W32" s="24" t="n"/>
     </row>
-    <row r="33" ht="20" customHeight="1">
+    <row r="33" ht="24" customHeight="1">
       <c r="A33" s="80" t="n"/>
       <c r="B33" s="80" t="n"/>
       <c r="C33" s="84" t="inlineStr">
@@ -4501,15 +4541,11 @@
       <c r="R33" s="83" t="n"/>
       <c r="S33" s="83" t="n"/>
       <c r="T33" s="83" t="n"/>
-      <c r="U33" s="138" t="inlineStr">
-        <is>
-          <t>Site JV</t>
-        </is>
-      </c>
-      <c r="V33" s="127" t="n"/>
+      <c r="U33" s="246" t="n"/>
+      <c r="V33" s="80" t="n"/>
       <c r="W33" s="24" t="n"/>
     </row>
-    <row r="34" ht="18" customHeight="1">
+    <row r="34" ht="19" customHeight="1">
       <c r="A34" s="80" t="n"/>
       <c r="B34" s="80" t="n"/>
       <c r="C34" s="108" t="inlineStr">
@@ -4559,14 +4595,10 @@
       <c r="R34" s="80" t="n"/>
       <c r="S34" s="80" t="n"/>
       <c r="T34" s="80" t="n"/>
-      <c r="U34" s="134" t="n"/>
-      <c r="V34" s="135" t="inlineStr">
-        <is>
-          <t>Cleanness</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="18" customHeight="1">
+      <c r="U34" s="80" t="n"/>
+      <c r="V34" s="245" t="n"/>
+    </row>
+    <row r="35" ht="19" customHeight="1">
       <c r="A35" s="80" t="n"/>
       <c r="B35" s="80" t="n"/>
       <c r="C35" s="113" t="n"/>
@@ -4608,14 +4640,10 @@
       <c r="R35" s="80" t="n"/>
       <c r="S35" s="80" t="n"/>
       <c r="T35" s="80" t="n"/>
-      <c r="U35" s="139" t="n"/>
-      <c r="V35" s="135" t="inlineStr">
-        <is>
-          <t>Over cement</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="18" customHeight="1">
+      <c r="U35" s="80" t="n"/>
+      <c r="V35" s="245" t="n"/>
+    </row>
+    <row r="36" ht="19" customHeight="1">
       <c r="A36" s="80" t="n"/>
       <c r="B36" s="80" t="n"/>
       <c r="C36" s="113" t="n"/>
@@ -4657,15 +4685,11 @@
       <c r="R36" s="83" t="n"/>
       <c r="S36" s="83" t="n"/>
       <c r="T36" s="83" t="n"/>
-      <c r="U36" s="136" t="n"/>
-      <c r="V36" s="129" t="inlineStr">
-        <is>
-          <t>Thread end</t>
-        </is>
-      </c>
+      <c r="U36" s="83" t="n"/>
+      <c r="V36" s="241" t="n"/>
       <c r="W36" s="24" t="n"/>
     </row>
-    <row r="37" ht="18" customHeight="1">
+    <row r="37" ht="19" customHeight="1">
       <c r="A37" s="80" t="n"/>
       <c r="B37" s="80" t="n"/>
       <c r="C37" s="113" t="n"/>
@@ -4707,12 +4731,8 @@
       <c r="R37" s="83" t="n"/>
       <c r="S37" s="83" t="n"/>
       <c r="T37" s="83" t="n"/>
-      <c r="U37" s="137" t="n"/>
-      <c r="V37" s="129" t="inlineStr">
-        <is>
-          <t>Sole attachment</t>
-        </is>
-      </c>
+      <c r="U37" s="83" t="n"/>
+      <c r="V37" s="241" t="n"/>
       <c r="W37" s="24" t="n"/>
     </row>
     <row r="38" ht="19" customHeight="1">
@@ -4761,7 +4781,7 @@
       <c r="V38" s="241" t="n"/>
       <c r="W38" s="24" t="n"/>
     </row>
-    <row r="39" ht="20" customHeight="1">
+    <row r="39" ht="24" customHeight="1">
       <c r="A39" s="80" t="n"/>
       <c r="B39" s="80" t="n"/>
       <c r="C39" s="84" t="inlineStr">
@@ -4827,22 +4847,18 @@
           <t>Heel/Tip height inconsistent</t>
         </is>
       </c>
-      <c r="R39" s="232" t="inlineStr">
+      <c r="R39" s="125" t="inlineStr">
         <is>
           <t>Rocking</t>
         </is>
       </c>
       <c r="S39" s="83" t="n"/>
       <c r="T39" s="83" t="n"/>
-      <c r="U39" s="138" t="inlineStr">
-        <is>
-          <t>Site JV2</t>
-        </is>
-      </c>
-      <c r="V39" s="127" t="n"/>
+      <c r="U39" s="246" t="n"/>
+      <c r="V39" s="80" t="n"/>
       <c r="W39" s="24" t="n"/>
     </row>
-    <row r="40" ht="18" customHeight="1">
+    <row r="40" ht="19" customHeight="1">
       <c r="A40" s="80" t="n"/>
       <c r="B40" s="80" t="n"/>
       <c r="C40" s="108" t="inlineStr">
@@ -4889,18 +4905,14 @@
       </c>
       <c r="P40" s="96" t="n"/>
       <c r="Q40" s="96" t="n"/>
-      <c r="R40" s="231" t="n"/>
+      <c r="R40" s="97" t="n"/>
       <c r="S40" s="83" t="n"/>
       <c r="T40" s="83" t="n"/>
-      <c r="U40" s="128" t="n"/>
-      <c r="V40" s="129" t="inlineStr">
-        <is>
-          <t>Cleanness</t>
-        </is>
-      </c>
+      <c r="U40" s="83" t="n"/>
+      <c r="V40" s="241" t="n"/>
       <c r="W40" s="24" t="n"/>
     </row>
-    <row r="41" ht="18" customHeight="1">
+    <row r="41" ht="19" customHeight="1">
       <c r="A41" s="80" t="n"/>
       <c r="B41" s="80" t="n"/>
       <c r="C41" s="113" t="n"/>
@@ -4939,17 +4951,13 @@
       <c r="Q41" s="123" t="n">
         <v>0.0912</v>
       </c>
-      <c r="R41" s="231" t="n"/>
+      <c r="R41" s="97" t="n"/>
       <c r="S41" s="80" t="n"/>
       <c r="T41" s="80" t="n"/>
-      <c r="U41" s="139" t="n"/>
-      <c r="V41" s="135" t="inlineStr">
-        <is>
-          <t>Over cement</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="18" customHeight="1">
+      <c r="U41" s="80" t="n"/>
+      <c r="V41" s="245" t="n"/>
+    </row>
+    <row r="42" ht="19" customHeight="1">
       <c r="A42" s="80" t="n"/>
       <c r="B42" s="80" t="n"/>
       <c r="C42" s="113" t="n"/>
@@ -4988,17 +4996,13 @@
       </c>
       <c r="P42" s="123" t="n"/>
       <c r="Q42" s="123" t="n"/>
-      <c r="R42" s="242" t="n"/>
+      <c r="R42" s="247" t="n"/>
       <c r="S42" s="80" t="n"/>
       <c r="T42" s="80" t="n"/>
-      <c r="U42" s="141" t="n"/>
-      <c r="V42" s="135" t="inlineStr">
-        <is>
-          <t>Thread end</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="18" customHeight="1">
+      <c r="U42" s="80" t="n"/>
+      <c r="V42" s="245" t="n"/>
+    </row>
+    <row r="43" ht="19" customHeight="1">
       <c r="A43" s="80" t="n"/>
       <c r="B43" s="80" t="n"/>
       <c r="C43" s="113" t="n"/>
@@ -5037,18 +5041,14 @@
         <v>0.094139</v>
       </c>
       <c r="Q43" s="96" t="n"/>
-      <c r="R43" s="231" t="n"/>
+      <c r="R43" s="97" t="n"/>
       <c r="S43" s="83" t="n"/>
       <c r="T43" s="83" t="n"/>
-      <c r="U43" s="142" t="n"/>
-      <c r="V43" s="129" t="inlineStr">
-        <is>
-          <t>Toe off center</t>
-        </is>
-      </c>
+      <c r="U43" s="83" t="n"/>
+      <c r="V43" s="241" t="n"/>
       <c r="W43" s="24" t="n"/>
     </row>
-    <row r="44" ht="18" customHeight="1">
+    <row r="44" ht="19" customHeight="1">
       <c r="A44" s="80" t="n"/>
       <c r="B44" s="80" t="n"/>
       <c r="C44" s="115" t="n"/>
@@ -5085,20 +5085,16 @@
       <c r="O44" s="119" t="n"/>
       <c r="P44" s="119" t="n"/>
       <c r="Q44" s="119" t="n"/>
-      <c r="R44" s="231" t="n">
+      <c r="R44" s="120" t="n">
         <v>0.084095</v>
       </c>
       <c r="S44" s="83" t="n"/>
       <c r="T44" s="83" t="n"/>
-      <c r="U44" s="243" t="n"/>
-      <c r="V44" s="129" t="inlineStr">
-        <is>
-          <t>Heel/Tip height inconsistent</t>
-        </is>
-      </c>
+      <c r="U44" s="83" t="n"/>
+      <c r="V44" s="241" t="n"/>
       <c r="W44" s="24" t="n"/>
     </row>
-    <row r="45" ht="15" customHeight="1">
+    <row r="45" ht="14" customHeight="1">
       <c r="A45" s="80" t="n"/>
       <c r="B45" s="80" t="n"/>
       <c r="C45" s="80" t="n"/>
@@ -5124,7 +5120,7 @@
       <c r="W45" s="83" t="n"/>
       <c r="X45" s="80" t="n"/>
     </row>
-    <row r="46" ht="15" customHeight="1">
+    <row r="46" ht="22" customHeight="1">
       <c r="A46" s="80" t="n"/>
       <c r="B46" s="80" t="n"/>
       <c r="C46" s="80" t="n"/>
@@ -5135,7 +5131,11 @@
       <c r="H46" s="80" t="n"/>
       <c r="I46" s="80" t="n"/>
       <c r="J46" s="80" t="n"/>
-      <c r="K46" s="80" t="n"/>
+      <c r="K46" s="248" t="inlineStr">
+        <is>
+          <t>Defect Color Legend by Factory (Jun, 2026)</t>
+        </is>
+      </c>
       <c r="L46" s="81" t="n"/>
       <c r="M46" s="82" t="n"/>
       <c r="N46" s="82" t="n"/>
@@ -5150,7 +5150,7 @@
       <c r="W46" s="83" t="n"/>
       <c r="X46" s="80" t="n"/>
     </row>
-    <row r="47" ht="15" customHeight="1">
+    <row r="47" ht="8" customHeight="1">
       <c r="A47" s="80" t="n"/>
       <c r="B47" s="80" t="n"/>
       <c r="C47" s="80" t="n"/>
@@ -5176,7 +5176,7 @@
       <c r="W47" s="83" t="n"/>
       <c r="X47" s="80" t="n"/>
     </row>
-    <row r="48" ht="15" customHeight="1">
+    <row r="48" ht="20" customHeight="1">
       <c r="A48" s="80" t="n"/>
       <c r="B48" s="80" t="n"/>
       <c r="C48" s="80" t="n"/>
@@ -5187,12 +5187,20 @@
       <c r="H48" s="80" t="n"/>
       <c r="I48" s="80" t="n"/>
       <c r="J48" s="80" t="n"/>
-      <c r="K48" s="80" t="n"/>
-      <c r="L48" s="80" t="n"/>
+      <c r="K48" s="126" t="inlineStr">
+        <is>
+          <t>Site VH</t>
+        </is>
+      </c>
+      <c r="L48" s="249" t="n"/>
       <c r="M48" s="80" t="n"/>
-      <c r="N48" s="80" t="n"/>
-      <c r="O48" s="80" t="n"/>
-      <c r="P48" s="80" t="n"/>
+      <c r="N48" s="126" t="inlineStr">
+        <is>
+          <t>Site VH2</t>
+        </is>
+      </c>
+      <c r="O48" s="249" t="n"/>
+      <c r="P48" s="249" t="n"/>
       <c r="Q48" s="80" t="n"/>
       <c r="R48" s="80" t="n"/>
       <c r="S48" s="80" t="n"/>
@@ -5202,7 +5210,7 @@
       <c r="W48" s="80" t="n"/>
       <c r="X48" s="80" t="n"/>
     </row>
-    <row r="49" ht="15" customHeight="1">
+    <row r="49" ht="18" customHeight="1">
       <c r="A49" s="80" t="n"/>
       <c r="B49" s="80" t="n"/>
       <c r="C49" s="80" t="n"/>
@@ -5213,12 +5221,20 @@
       <c r="H49" s="80" t="n"/>
       <c r="I49" s="80" t="n"/>
       <c r="J49" s="80" t="n"/>
-      <c r="K49" s="80" t="n"/>
-      <c r="L49" s="80" t="n"/>
+      <c r="K49" s="134" t="n"/>
+      <c r="L49" s="135" t="inlineStr">
+        <is>
+          <t>Cleanness</t>
+        </is>
+      </c>
       <c r="M49" s="80" t="n"/>
-      <c r="N49" s="80" t="n"/>
-      <c r="O49" s="80" t="n"/>
-      <c r="P49" s="80" t="n"/>
+      <c r="N49" s="134" t="n"/>
+      <c r="O49" s="135" t="inlineStr">
+        <is>
+          <t>Cleanness</t>
+        </is>
+      </c>
+      <c r="P49" s="127" t="n"/>
       <c r="Q49" s="80" t="n"/>
       <c r="R49" s="80" t="n"/>
       <c r="S49" s="80" t="n"/>
@@ -5228,7 +5244,7 @@
       <c r="W49" s="80" t="n"/>
       <c r="X49" s="80" t="n"/>
     </row>
-    <row r="50" ht="15" customHeight="1">
+    <row r="50" ht="18" customHeight="1">
       <c r="A50" s="80" t="n"/>
       <c r="B50" s="80" t="n"/>
       <c r="C50" s="80" t="n"/>
@@ -5239,12 +5255,20 @@
       <c r="H50" s="80" t="n"/>
       <c r="I50" s="80" t="n"/>
       <c r="J50" s="80" t="n"/>
-      <c r="K50" s="80" t="n"/>
-      <c r="L50" s="80" t="n"/>
+      <c r="K50" s="139" t="n"/>
+      <c r="L50" s="135" t="inlineStr">
+        <is>
+          <t>Over cement</t>
+        </is>
+      </c>
       <c r="M50" s="80" t="n"/>
-      <c r="N50" s="80" t="n"/>
-      <c r="O50" s="80" t="n"/>
-      <c r="P50" s="80" t="n"/>
+      <c r="N50" s="141" t="n"/>
+      <c r="O50" s="135" t="inlineStr">
+        <is>
+          <t>Thread end</t>
+        </is>
+      </c>
+      <c r="P50" s="127" t="n"/>
       <c r="Q50" s="80" t="n"/>
       <c r="R50" s="80" t="n"/>
       <c r="S50" s="80" t="n"/>
@@ -5254,7 +5278,7 @@
       <c r="W50" s="80" t="n"/>
       <c r="X50" s="80" t="n"/>
     </row>
-    <row r="51" ht="15" customHeight="1">
+    <row r="51" ht="18" customHeight="1">
       <c r="A51" s="80" t="n"/>
       <c r="B51" s="80" t="n"/>
       <c r="C51" s="80" t="n"/>
@@ -5265,12 +5289,20 @@
       <c r="H51" s="80" t="n"/>
       <c r="I51" s="80" t="n"/>
       <c r="J51" s="80" t="n"/>
-      <c r="K51" s="80" t="n"/>
-      <c r="L51" s="80" t="n"/>
+      <c r="K51" s="250" t="n"/>
+      <c r="L51" s="135" t="inlineStr">
+        <is>
+          <t>Rocking</t>
+        </is>
+      </c>
       <c r="M51" s="80" t="n"/>
-      <c r="N51" s="80" t="n"/>
-      <c r="O51" s="80" t="n"/>
-      <c r="P51" s="80" t="n"/>
+      <c r="N51" s="139" t="n"/>
+      <c r="O51" s="135" t="inlineStr">
+        <is>
+          <t>Over cement</t>
+        </is>
+      </c>
+      <c r="P51" s="127" t="n"/>
       <c r="Q51" s="80" t="n"/>
       <c r="R51" s="80" t="n"/>
       <c r="S51" s="80" t="n"/>
@@ -5280,7 +5312,7 @@
       <c r="W51" s="80" t="n"/>
       <c r="X51" s="80" t="n"/>
     </row>
-    <row r="52" ht="15" customHeight="1">
+    <row r="52" ht="18" customHeight="1">
       <c r="A52" s="80" t="n"/>
       <c r="B52" s="80" t="n"/>
       <c r="C52" s="80" t="n"/>
@@ -5291,12 +5323,20 @@
       <c r="H52" s="80" t="n"/>
       <c r="I52" s="80" t="n"/>
       <c r="J52" s="80" t="n"/>
-      <c r="K52" s="80" t="n"/>
-      <c r="L52" s="80" t="n"/>
+      <c r="K52" s="141" t="n"/>
+      <c r="L52" s="135" t="inlineStr">
+        <is>
+          <t>Thread end</t>
+        </is>
+      </c>
       <c r="M52" s="80" t="n"/>
-      <c r="N52" s="80" t="n"/>
-      <c r="O52" s="80" t="n"/>
-      <c r="P52" s="80" t="n"/>
+      <c r="N52" s="251" t="n"/>
+      <c r="O52" s="135" t="inlineStr">
+        <is>
+          <t>Airbag quality/stain</t>
+        </is>
+      </c>
+      <c r="P52" s="127" t="n"/>
       <c r="Q52" s="80" t="n"/>
       <c r="R52" s="80" t="n"/>
       <c r="S52" s="80" t="n"/>
@@ -5306,7 +5346,7 @@
       <c r="W52" s="80" t="n"/>
       <c r="X52" s="80" t="n"/>
     </row>
-    <row r="53" ht="15" customHeight="1">
+    <row r="53" ht="18" customHeight="1">
       <c r="A53" s="80" t="n"/>
       <c r="B53" s="80" t="n"/>
       <c r="C53" s="80" t="n"/>
@@ -5317,12 +5357,20 @@
       <c r="H53" s="80" t="n"/>
       <c r="I53" s="80" t="n"/>
       <c r="J53" s="80" t="n"/>
-      <c r="K53" s="80" t="n"/>
-      <c r="L53" s="80" t="n"/>
+      <c r="K53" s="252" t="n"/>
+      <c r="L53" s="135" t="inlineStr">
+        <is>
+          <t>Components inconsistent</t>
+        </is>
+      </c>
       <c r="M53" s="80" t="n"/>
-      <c r="N53" s="80" t="n"/>
-      <c r="O53" s="80" t="n"/>
-      <c r="P53" s="80" t="n"/>
+      <c r="N53" s="253" t="n"/>
+      <c r="O53" s="135" t="inlineStr">
+        <is>
+          <t>Midsole/Outsole to upper bond gap</t>
+        </is>
+      </c>
+      <c r="P53" s="127" t="n"/>
       <c r="Q53" s="80" t="n"/>
       <c r="R53" s="80" t="n"/>
       <c r="S53" s="80" t="n"/>
@@ -5332,7 +5380,7 @@
       <c r="W53" s="80" t="n"/>
       <c r="X53" s="80" t="n"/>
     </row>
-    <row r="54" ht="15" customHeight="1">
+    <row r="54" ht="18" customHeight="1">
       <c r="A54" s="80" t="n"/>
       <c r="B54" s="80" t="n"/>
       <c r="C54" s="80" t="n"/>
@@ -5343,8 +5391,12 @@
       <c r="H54" s="80" t="n"/>
       <c r="I54" s="80" t="n"/>
       <c r="J54" s="80" t="n"/>
-      <c r="K54" s="80" t="n"/>
-      <c r="L54" s="80" t="n"/>
+      <c r="K54" s="253" t="n"/>
+      <c r="L54" s="135" t="inlineStr">
+        <is>
+          <t>Midsole/Outsole to upper bond gap</t>
+        </is>
+      </c>
       <c r="M54" s="80" t="n"/>
       <c r="N54" s="80" t="n"/>
       <c r="O54" s="80" t="n"/>
@@ -5358,7 +5410,7 @@
       <c r="W54" s="80" t="n"/>
       <c r="X54" s="80" t="n"/>
     </row>
-    <row r="55" ht="15" customHeight="1">
+    <row r="55" ht="16" customHeight="1">
       <c r="A55" s="80" t="n"/>
       <c r="B55" s="80" t="n"/>
       <c r="C55" s="80" t="n"/>
@@ -5384,7 +5436,7 @@
       <c r="W55" s="80" t="n"/>
       <c r="X55" s="80" t="n"/>
     </row>
-    <row r="56" ht="15" customHeight="1">
+    <row r="56" ht="20" customHeight="1">
       <c r="A56" s="80" t="n"/>
       <c r="B56" s="80" t="n"/>
       <c r="C56" s="80" t="n"/>
@@ -5395,12 +5447,20 @@
       <c r="H56" s="80" t="n"/>
       <c r="I56" s="80" t="n"/>
       <c r="J56" s="80" t="n"/>
-      <c r="K56" s="80" t="n"/>
-      <c r="L56" s="80" t="n"/>
+      <c r="K56" s="126" t="inlineStr">
+        <is>
+          <t>Site JV</t>
+        </is>
+      </c>
+      <c r="L56" s="249" t="n"/>
       <c r="M56" s="80" t="n"/>
-      <c r="N56" s="80" t="n"/>
-      <c r="O56" s="80" t="n"/>
-      <c r="P56" s="80" t="n"/>
+      <c r="N56" s="126" t="inlineStr">
+        <is>
+          <t>Site JV2</t>
+        </is>
+      </c>
+      <c r="O56" s="249" t="n"/>
+      <c r="P56" s="249" t="n"/>
       <c r="Q56" s="80" t="n"/>
       <c r="R56" s="80" t="n"/>
       <c r="S56" s="80" t="n"/>
@@ -5410,7 +5470,7 @@
       <c r="W56" s="80" t="n"/>
       <c r="X56" s="80" t="n"/>
     </row>
-    <row r="57" ht="15" customHeight="1">
+    <row r="57" ht="18" customHeight="1">
       <c r="A57" s="80" t="n"/>
       <c r="B57" s="80" t="n"/>
       <c r="C57" s="80" t="n"/>
@@ -5421,12 +5481,20 @@
       <c r="H57" s="80" t="n"/>
       <c r="I57" s="80" t="n"/>
       <c r="J57" s="80" t="n"/>
-      <c r="K57" s="80" t="n"/>
-      <c r="L57" s="80" t="n"/>
+      <c r="K57" s="134" t="n"/>
+      <c r="L57" s="135" t="inlineStr">
+        <is>
+          <t>Cleanness</t>
+        </is>
+      </c>
       <c r="M57" s="80" t="n"/>
-      <c r="N57" s="80" t="n"/>
-      <c r="O57" s="80" t="n"/>
-      <c r="P57" s="80" t="n"/>
+      <c r="N57" s="134" t="n"/>
+      <c r="O57" s="135" t="inlineStr">
+        <is>
+          <t>Cleanness</t>
+        </is>
+      </c>
+      <c r="P57" s="127" t="n"/>
       <c r="Q57" s="80" t="n"/>
       <c r="R57" s="80" t="n"/>
       <c r="S57" s="80" t="n"/>
@@ -5436,7 +5504,7 @@
       <c r="W57" s="80" t="n"/>
       <c r="X57" s="80" t="n"/>
     </row>
-    <row r="58" ht="15" customHeight="1">
+    <row r="58" ht="18" customHeight="1">
       <c r="A58" s="80" t="n"/>
       <c r="B58" s="80" t="n"/>
       <c r="C58" s="80" t="n"/>
@@ -5447,12 +5515,20 @@
       <c r="H58" s="80" t="n"/>
       <c r="I58" s="80" t="n"/>
       <c r="J58" s="80" t="n"/>
-      <c r="K58" s="80" t="n"/>
-      <c r="L58" s="80" t="n"/>
+      <c r="K58" s="139" t="n"/>
+      <c r="L58" s="135" t="inlineStr">
+        <is>
+          <t>Over cement</t>
+        </is>
+      </c>
       <c r="M58" s="80" t="n"/>
-      <c r="N58" s="80" t="n"/>
-      <c r="O58" s="80" t="n"/>
-      <c r="P58" s="80" t="n"/>
+      <c r="N58" s="139" t="n"/>
+      <c r="O58" s="135" t="inlineStr">
+        <is>
+          <t>Over cement</t>
+        </is>
+      </c>
+      <c r="P58" s="127" t="n"/>
       <c r="Q58" s="80" t="n"/>
       <c r="R58" s="80" t="n"/>
       <c r="S58" s="80" t="n"/>
@@ -5462,7 +5538,7 @@
       <c r="W58" s="80" t="n"/>
       <c r="X58" s="80" t="n"/>
     </row>
-    <row r="59" ht="15" customHeight="1">
+    <row r="59" ht="18" customHeight="1">
       <c r="A59" s="80" t="n"/>
       <c r="B59" s="80" t="n"/>
       <c r="C59" s="80" t="n"/>
@@ -5473,12 +5549,20 @@
       <c r="H59" s="80" t="n"/>
       <c r="I59" s="80" t="n"/>
       <c r="J59" s="80" t="n"/>
-      <c r="K59" s="80" t="n"/>
-      <c r="L59" s="80" t="n"/>
+      <c r="K59" s="141" t="n"/>
+      <c r="L59" s="135" t="inlineStr">
+        <is>
+          <t>Thread end</t>
+        </is>
+      </c>
       <c r="M59" s="80" t="n"/>
-      <c r="N59" s="80" t="n"/>
-      <c r="O59" s="80" t="n"/>
-      <c r="P59" s="80" t="n"/>
+      <c r="N59" s="141" t="n"/>
+      <c r="O59" s="135" t="inlineStr">
+        <is>
+          <t>Thread end</t>
+        </is>
+      </c>
+      <c r="P59" s="127" t="n"/>
       <c r="Q59" s="80" t="n"/>
       <c r="R59" s="80" t="n"/>
       <c r="S59" s="80" t="n"/>
@@ -5488,7 +5572,7 @@
       <c r="W59" s="80" t="n"/>
       <c r="X59" s="80" t="n"/>
     </row>
-    <row r="60" ht="15" customHeight="1">
+    <row r="60" ht="18" customHeight="1">
       <c r="A60" s="80" t="n"/>
       <c r="B60" s="80" t="n"/>
       <c r="C60" s="80" t="n"/>
@@ -5499,12 +5583,20 @@
       <c r="H60" s="80" t="n"/>
       <c r="I60" s="80" t="n"/>
       <c r="J60" s="80" t="n"/>
-      <c r="K60" s="80" t="n"/>
-      <c r="L60" s="80" t="n"/>
+      <c r="K60" s="254" t="n"/>
+      <c r="L60" s="135" t="inlineStr">
+        <is>
+          <t>Sole attachment</t>
+        </is>
+      </c>
       <c r="M60" s="80" t="n"/>
-      <c r="N60" s="80" t="n"/>
-      <c r="O60" s="80" t="n"/>
-      <c r="P60" s="80" t="n"/>
+      <c r="N60" s="255" t="n"/>
+      <c r="O60" s="135" t="inlineStr">
+        <is>
+          <t>Toe off center</t>
+        </is>
+      </c>
+      <c r="P60" s="127" t="n"/>
       <c r="Q60" s="80" t="n"/>
       <c r="R60" s="80" t="n"/>
       <c r="S60" s="80" t="n"/>
@@ -5514,7 +5606,7 @@
       <c r="W60" s="80" t="n"/>
       <c r="X60" s="80" t="n"/>
     </row>
-    <row r="61" ht="15" customHeight="1">
+    <row r="61" ht="18" customHeight="1">
       <c r="A61" s="80" t="n"/>
       <c r="B61" s="80" t="n"/>
       <c r="C61" s="80" t="n"/>
@@ -5528,9 +5620,13 @@
       <c r="K61" s="80" t="n"/>
       <c r="L61" s="80" t="n"/>
       <c r="M61" s="80" t="n"/>
-      <c r="N61" s="80" t="n"/>
-      <c r="O61" s="80" t="n"/>
-      <c r="P61" s="80" t="n"/>
+      <c r="N61" s="256" t="n"/>
+      <c r="O61" s="135" t="inlineStr">
+        <is>
+          <t>Heel/Tip height inconsistent</t>
+        </is>
+      </c>
+      <c r="P61" s="127" t="n"/>
       <c r="Q61" s="80" t="n"/>
       <c r="R61" s="80" t="n"/>
       <c r="S61" s="80" t="n"/>
@@ -5540,7 +5636,7 @@
       <c r="W61" s="80" t="n"/>
       <c r="X61" s="80" t="n"/>
     </row>
-    <row r="62" ht="15" customHeight="1">
+    <row r="62" ht="18" customHeight="1">
       <c r="A62" s="80" t="n"/>
       <c r="B62" s="80" t="n"/>
       <c r="C62" s="80" t="n"/>
@@ -5554,9 +5650,13 @@
       <c r="K62" s="80" t="n"/>
       <c r="L62" s="80" t="n"/>
       <c r="M62" s="80" t="n"/>
-      <c r="N62" s="80" t="n"/>
-      <c r="O62" s="80" t="n"/>
-      <c r="P62" s="80" t="n"/>
+      <c r="N62" s="250" t="n"/>
+      <c r="O62" s="135" t="inlineStr">
+        <is>
+          <t>Rocking</t>
+        </is>
+      </c>
+      <c r="P62" s="127" t="n"/>
       <c r="Q62" s="80" t="n"/>
       <c r="R62" s="80" t="n"/>
       <c r="S62" s="80" t="n"/>
@@ -5566,7 +5666,7 @@
       <c r="W62" s="80" t="n"/>
       <c r="X62" s="80" t="n"/>
     </row>
-    <row r="63" ht="15" customHeight="1">
+    <row r="63" ht="16" customHeight="1">
       <c r="A63" s="80" t="n"/>
       <c r="B63" s="80" t="n"/>
       <c r="C63" s="80" t="n"/>
@@ -5592,7 +5692,7 @@
       <c r="W63" s="80" t="n"/>
       <c r="X63" s="80" t="n"/>
     </row>
-    <row r="64" ht="15" customHeight="1">
+    <row r="64" ht="16" customHeight="1">
       <c r="A64" s="80" t="n"/>
       <c r="B64" s="80" t="n"/>
       <c r="C64" s="80" t="n"/>
@@ -5618,20 +5718,57 @@
       <c r="W64" s="80" t="n"/>
       <c r="X64" s="80" t="n"/>
     </row>
+    <row r="65" ht="16" customHeight="1">
+      <c r="A65" s="80" t="n"/>
+      <c r="B65" s="80" t="n"/>
+      <c r="C65" s="80" t="n"/>
+      <c r="D65" s="80" t="n"/>
+      <c r="E65" s="80" t="n"/>
+      <c r="F65" s="80" t="n"/>
+      <c r="G65" s="80" t="n"/>
+      <c r="H65" s="80" t="n"/>
+      <c r="I65" s="80" t="n"/>
+      <c r="J65" s="80" t="n"/>
+      <c r="K65" s="80" t="n"/>
+      <c r="L65" s="80" t="n"/>
+      <c r="M65" s="80" t="n"/>
+      <c r="N65" s="80" t="n"/>
+      <c r="O65" s="80" t="n"/>
+      <c r="P65" s="80" t="n"/>
+      <c r="Q65" s="80" t="n"/>
+      <c r="R65" s="80" t="n"/>
+      <c r="S65" s="80" t="n"/>
+      <c r="T65" s="80" t="n"/>
+      <c r="U65" s="80" t="n"/>
+      <c r="V65" s="80" t="n"/>
+      <c r="W65" s="80" t="n"/>
+      <c r="X65" s="80" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="23">
     <mergeCell ref="C40:C44"/>
-    <mergeCell ref="C22:C26"/>
+    <mergeCell ref="O53:P53"/>
+    <mergeCell ref="N48:P48"/>
+    <mergeCell ref="O49:P49"/>
+    <mergeCell ref="C28:C32"/>
+    <mergeCell ref="K28:K32"/>
+    <mergeCell ref="K56:L56"/>
     <mergeCell ref="C34:C38"/>
     <mergeCell ref="K34:K38"/>
-    <mergeCell ref="U21:V21"/>
-    <mergeCell ref="U33:V33"/>
-    <mergeCell ref="C28:C32"/>
-    <mergeCell ref="K28:K32"/>
-    <mergeCell ref="U27:V27"/>
+    <mergeCell ref="O59:P59"/>
+    <mergeCell ref="O50:P50"/>
+    <mergeCell ref="O51:P51"/>
+    <mergeCell ref="O62:P62"/>
+    <mergeCell ref="O61:P61"/>
+    <mergeCell ref="O58:P58"/>
+    <mergeCell ref="K48:L48"/>
+    <mergeCell ref="O52:P52"/>
+    <mergeCell ref="O60:P60"/>
+    <mergeCell ref="N56:P56"/>
+    <mergeCell ref="O57:P57"/>
+    <mergeCell ref="C22:C26"/>
     <mergeCell ref="K22:K26"/>
     <mergeCell ref="K40:K44"/>
-    <mergeCell ref="U39:V39"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>

</xml_diff>

<commit_message>
feat: update reconciliation pipeline, pptx annotator, agents and latest input data
</commit_message>
<xml_diff>
--- a/Database/HFPA_Template.xlsx
+++ b/Database/HFPA_Template.xlsx
@@ -326,7 +326,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="122">
+  <fills count="130">
     <fill>
       <patternFill/>
     </fill>
@@ -1051,6 +1051,54 @@
       <patternFill patternType="solid">
         <fgColor rgb="00336A4E"/>
         <bgColor rgb="00336A4E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00770BE1"/>
+        <bgColor rgb="00770BE1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0000B050"/>
+        <bgColor rgb="0000B050"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000070C0"/>
+        <bgColor rgb="000070C0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="003CE263"/>
+        <bgColor rgb="003CE263"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D980FA"/>
+        <bgColor rgb="00D980FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FE9BFF"/>
+        <bgColor rgb="00FE9BFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C19A6B"/>
+        <bgColor rgb="00C19A6B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FAC090"/>
+        <bgColor rgb="00FAC090"/>
       </patternFill>
     </fill>
   </fills>
@@ -1714,7 +1762,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="257">
+  <cellXfs count="269">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -2368,6 +2416,22 @@
     <xf numFmtId="0" fontId="0" fillId="47" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="49" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="121" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="119" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="33" fillId="38" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="123" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="122" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="124" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="125" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="126" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="127" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="128" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="129" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="48" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="50">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2926,7 +2990,9 @@
       <c r="J2" s="90" t="n">
         <v>252237</v>
       </c>
-      <c r="K2" s="90" t="n"/>
+      <c r="K2" s="90" t="n">
+        <v>191303</v>
+      </c>
       <c r="L2" s="90" t="n"/>
       <c r="M2" s="90" t="n"/>
       <c r="N2" s="91" t="n"/>
@@ -2968,7 +3034,9 @@
       <c r="J3" s="90" t="n">
         <v>187637</v>
       </c>
-      <c r="K3" s="90" t="n"/>
+      <c r="K3" s="90" t="n">
+        <v>175514</v>
+      </c>
       <c r="L3" s="90" t="n"/>
       <c r="M3" s="90" t="n"/>
       <c r="N3" s="91" t="n"/>
@@ -3010,7 +3078,9 @@
       <c r="J4" s="90" t="n">
         <v>92175</v>
       </c>
-      <c r="K4" s="90" t="n"/>
+      <c r="K4" s="90" t="n">
+        <v>97919</v>
+      </c>
       <c r="L4" s="90" t="n"/>
       <c r="M4" s="90" t="n"/>
       <c r="N4" s="91" t="n"/>
@@ -3052,7 +3122,9 @@
       <c r="J5" s="90" t="n">
         <v>76104</v>
       </c>
-      <c r="K5" s="90" t="n"/>
+      <c r="K5" s="90" t="n">
+        <v>79079</v>
+      </c>
       <c r="L5" s="90" t="n"/>
       <c r="M5" s="90" t="n"/>
       <c r="N5" s="91" t="n"/>
@@ -3257,7 +3329,9 @@
       <c r="J9" s="90" t="n">
         <v>40405</v>
       </c>
-      <c r="K9" s="90" t="n"/>
+      <c r="K9" s="90" t="n">
+        <v>30535</v>
+      </c>
       <c r="L9" s="90" t="n"/>
       <c r="M9" s="90" t="n"/>
       <c r="N9" s="91" t="n"/>
@@ -3299,7 +3373,9 @@
       <c r="J10" s="90" t="n">
         <v>27355</v>
       </c>
-      <c r="K10" s="90" t="n"/>
+      <c r="K10" s="90" t="n">
+        <v>25464</v>
+      </c>
       <c r="L10" s="90" t="n"/>
       <c r="M10" s="90" t="n"/>
       <c r="N10" s="91" t="n"/>
@@ -3341,7 +3417,9 @@
       <c r="J11" s="90" t="n">
         <v>11421</v>
       </c>
-      <c r="K11" s="90" t="n"/>
+      <c r="K11" s="90" t="n">
+        <v>12584</v>
+      </c>
       <c r="L11" s="90" t="n"/>
       <c r="M11" s="90" t="n"/>
       <c r="N11" s="91" t="n"/>
@@ -3383,7 +3461,9 @@
       <c r="J12" s="90" t="n">
         <v>4503</v>
       </c>
-      <c r="K12" s="90" t="n"/>
+      <c r="K12" s="90" t="n">
+        <v>4580</v>
+      </c>
       <c r="L12" s="90" t="n"/>
       <c r="M12" s="90" t="n"/>
       <c r="N12" s="91" t="n"/>
@@ -3837,7 +3917,10 @@
         <f>IF(J6&gt;0, 1-J13/J6, "")</f>
         <v/>
       </c>
-      <c r="K20" s="98" t="n"/>
+      <c r="K20" s="258">
+        <f>IF(K6&gt;0, 1-K13/K6, "")</f>
+        <v/>
+      </c>
       <c r="L20" s="98" t="n"/>
       <c r="M20" s="98" t="n"/>
       <c r="N20" s="101" t="n"/>
@@ -3849,7 +3932,7 @@
       <c r="A21" s="80" t="n"/>
       <c r="B21" s="102" t="inlineStr">
         <is>
-          <t>Top 5 model (Jun, 2026)</t>
+          <t>Top 5 model (Sep, 2026)</t>
         </is>
       </c>
       <c r="C21" s="84" t="inlineStr">
@@ -3881,7 +3964,7 @@
       <c r="I21" s="103" t="n"/>
       <c r="J21" s="104" t="inlineStr">
         <is>
-          <t>Top 5 defect (Jun, 2026)</t>
+          <t>Top 5 defect (Sep, 2026)</t>
         </is>
       </c>
       <c r="K21" s="105" t="inlineStr">
@@ -3906,25 +3989,25 @@
       </c>
       <c r="O21" s="106" t="inlineStr">
         <is>
-          <t>Rocking</t>
+          <t>Components inconsistent</t>
         </is>
       </c>
       <c r="P21" s="106" t="inlineStr">
         <is>
-          <t>Thread end</t>
+          <t>Heel/Tip height inconsistent</t>
         </is>
       </c>
       <c r="Q21" s="106" t="inlineStr">
         <is>
-          <t>Components inconsistent</t>
+          <t>Wrinkle bottom</t>
         </is>
       </c>
       <c r="R21" s="107" t="inlineStr">
         <is>
-          <t>Midsole/Outsole to upper bond gap</t>
-        </is>
-      </c>
-      <c r="S21" s="80" t="n"/>
+          <t>Over buffing</t>
+        </is>
+      </c>
+      <c r="S21" s="230" t="n"/>
       <c r="T21" s="80" t="n"/>
       <c r="U21" s="244" t="n"/>
       <c r="V21" s="80" t="n"/>
@@ -3939,14 +4022,14 @@
       </c>
       <c r="D22" s="89" t="inlineStr">
         <is>
-          <t>NIKE AIR WINFLO 12 (MS/WS)</t>
+          <t>NIKE SB FORCE 58</t>
         </is>
       </c>
       <c r="E22" s="90" t="n">
-        <v>229614</v>
+        <v>191303</v>
       </c>
       <c r="F22" s="90" t="n">
-        <v>3512</v>
+        <v>1982</v>
       </c>
       <c r="G22" s="109">
         <f>F22/E22</f>
@@ -3962,22 +4045,22 @@
       </c>
       <c r="L22" s="89" t="inlineStr">
         <is>
-          <t>NIKE AIR WINFLO 12 (MS/WS)</t>
+          <t>NIKE SB FORCE 58</t>
         </is>
       </c>
       <c r="M22" s="96" t="n">
-        <v>0.146748</v>
+        <v>0.231505</v>
       </c>
       <c r="N22" s="96" t="n">
-        <v>0.129491</v>
-      </c>
-      <c r="O22" s="96" t="n"/>
-      <c r="P22" s="96" t="n">
-        <v>0.097844</v>
-      </c>
+        <v>0.242073</v>
+      </c>
+      <c r="O22" s="96" t="n">
+        <v>0.117262</v>
+      </c>
+      <c r="P22" s="96" t="n"/>
       <c r="Q22" s="96" t="n"/>
       <c r="R22" s="97" t="n"/>
-      <c r="S22" s="83" t="n"/>
+      <c r="S22" s="231" t="n"/>
       <c r="T22" s="83" t="n"/>
       <c r="U22" s="83" t="n"/>
       <c r="V22" s="241" t="n"/>
@@ -3989,14 +4072,14 @@
       <c r="C23" s="113" t="n"/>
       <c r="D23" s="89" t="inlineStr">
         <is>
-          <t>JORDAN SPIZIKE LOW (GS)</t>
+          <t>NIKE MANOA LEATHER</t>
         </is>
       </c>
       <c r="E23" s="90" t="n">
-        <v>229614</v>
+        <v>191303</v>
       </c>
       <c r="F23" s="90" t="n">
-        <v>2379</v>
+        <v>1786</v>
       </c>
       <c r="G23" s="109">
         <f>F23/E23</f>
@@ -4008,22 +4091,22 @@
       <c r="K23" s="113" t="n"/>
       <c r="L23" s="89" t="inlineStr">
         <is>
-          <t>JORDAN SPIZIKE LOW (GS)</t>
+          <t>NIKE MANOA LEATHER</t>
         </is>
       </c>
       <c r="M23" s="96" t="n">
-        <v>0.180101</v>
+        <v>0.174399</v>
       </c>
       <c r="N23" s="96" t="n">
-        <v>0.143577</v>
+        <v>0.137507</v>
       </c>
       <c r="O23" s="96" t="n"/>
-      <c r="P23" s="96" t="n">
-        <v>0.154912</v>
-      </c>
+      <c r="P23" s="96" t="n"/>
       <c r="Q23" s="96" t="n"/>
-      <c r="R23" s="97" t="n"/>
-      <c r="S23" s="83" t="n"/>
+      <c r="R23" s="97" t="n">
+        <v>0.09837899999999999</v>
+      </c>
+      <c r="S23" s="231" t="n"/>
       <c r="T23" s="83" t="n"/>
       <c r="U23" s="83" t="n"/>
       <c r="V23" s="241" t="n"/>
@@ -4035,14 +4118,14 @@
       <c r="C24" s="113" t="n"/>
       <c r="D24" s="89" t="inlineStr">
         <is>
-          <t>NIKE SB FORCE 58</t>
+          <t>WMNS BENASSI JDI</t>
         </is>
       </c>
       <c r="E24" s="90" t="n">
-        <v>229614</v>
+        <v>191303</v>
       </c>
       <c r="F24" s="90" t="n">
-        <v>2171</v>
+        <v>1515</v>
       </c>
       <c r="G24" s="109">
         <f>F24/E24</f>
@@ -4054,22 +4137,22 @@
       <c r="K24" s="113" t="n"/>
       <c r="L24" s="89" t="inlineStr">
         <is>
-          <t>NIKE SB FORCE 58</t>
+          <t>WMNS BENASSI JDI</t>
         </is>
       </c>
       <c r="M24" s="96" t="n">
-        <v>0.220952</v>
+        <v>0.164248</v>
       </c>
       <c r="N24" s="96" t="n">
-        <v>0.23513</v>
+        <v>0.141821</v>
       </c>
       <c r="O24" s="96" t="n"/>
-      <c r="P24" s="96" t="n"/>
-      <c r="Q24" s="96" t="n">
-        <v>0.126007</v>
-      </c>
+      <c r="P24" s="96" t="n">
+        <v>0.120712</v>
+      </c>
+      <c r="Q24" s="96" t="n"/>
       <c r="R24" s="97" t="n"/>
-      <c r="S24" s="83" t="n"/>
+      <c r="S24" s="231" t="n"/>
       <c r="T24" s="83" t="n"/>
       <c r="U24" s="83" t="n"/>
       <c r="V24" s="241" t="n"/>
@@ -4081,14 +4164,14 @@
       <c r="C25" s="113" t="n"/>
       <c r="D25" s="89" t="inlineStr">
         <is>
-          <t>AIR JORDAN 1 LOW SE (MS/WS)</t>
+          <t>JORDAN TRUE FLIGHT (MS)</t>
         </is>
       </c>
       <c r="E25" s="90" t="n">
-        <v>229614</v>
+        <v>191303</v>
       </c>
       <c r="F25" s="90" t="n">
-        <v>1651</v>
+        <v>1309</v>
       </c>
       <c r="G25" s="109">
         <f>F25/E25</f>
@@ -4100,22 +4183,22 @@
       <c r="K25" s="113" t="n"/>
       <c r="L25" s="89" t="inlineStr">
         <is>
-          <t>AIR JORDAN 1 LOW SE (MS/WS)</t>
+          <t>JORDAN TRUE FLIGHT (MS)</t>
         </is>
       </c>
       <c r="M25" s="96" t="n">
-        <v>0.172078</v>
+        <v>0.156012</v>
       </c>
       <c r="N25" s="96" t="n">
-        <v>0.168405</v>
-      </c>
-      <c r="O25" s="96" t="n">
-        <v>0.126276</v>
-      </c>
+        <v>0.11035</v>
+      </c>
+      <c r="O25" s="96" t="n"/>
       <c r="P25" s="96" t="n"/>
-      <c r="Q25" s="96" t="n"/>
+      <c r="Q25" s="96" t="n">
+        <v>0.101979</v>
+      </c>
       <c r="R25" s="97" t="n"/>
-      <c r="S25" s="83" t="n"/>
+      <c r="S25" s="231" t="n"/>
       <c r="T25" s="83" t="n"/>
       <c r="U25" s="83" t="n"/>
       <c r="V25" s="241" t="n"/>
@@ -4127,14 +4210,14 @@
       <c r="C26" s="115" t="n"/>
       <c r="D26" s="116" t="inlineStr">
         <is>
-          <t>WMNS BENASSI JDI</t>
+          <t>AIR JORDAN 1 LOW SE (MS/WS)</t>
         </is>
       </c>
       <c r="E26" s="117" t="n">
-        <v>229614</v>
+        <v>191303</v>
       </c>
       <c r="F26" s="117" t="n">
-        <v>1409</v>
+        <v>1275</v>
       </c>
       <c r="G26" s="118">
         <f>F26/E26</f>
@@ -4146,22 +4229,22 @@
       <c r="K26" s="115" t="n"/>
       <c r="L26" s="116" t="inlineStr">
         <is>
-          <t>WMNS BENASSI JDI</t>
+          <t>AIR JORDAN 1 LOW SE (MS/WS)</t>
         </is>
       </c>
       <c r="M26" s="119" t="n">
-        <v>0.206529</v>
-      </c>
-      <c r="N26" s="119" t="n"/>
+        <v>0.222048</v>
+      </c>
+      <c r="N26" s="119" t="n">
+        <v>0.203284</v>
+      </c>
       <c r="O26" s="119" t="n">
-        <v>0.149752</v>
+        <v>0.148554</v>
       </c>
       <c r="P26" s="119" t="n"/>
       <c r="Q26" s="119" t="n"/>
-      <c r="R26" s="120" t="n">
-        <v>0.125621</v>
-      </c>
-      <c r="S26" s="83" t="n"/>
+      <c r="R26" s="120" t="n"/>
+      <c r="S26" s="231" t="n"/>
       <c r="T26" s="83" t="n"/>
       <c r="U26" s="83" t="n"/>
       <c r="V26" s="241" t="n"/>
@@ -4215,24 +4298,20 @@
       </c>
       <c r="N27" s="122" t="inlineStr">
         <is>
+          <t>Over cement</t>
+        </is>
+      </c>
+      <c r="O27" s="106" t="inlineStr">
+        <is>
           <t>Thread end</t>
         </is>
       </c>
-      <c r="O27" s="106" t="inlineStr">
-        <is>
-          <t>Over cement</t>
-        </is>
-      </c>
-      <c r="P27" s="122" t="inlineStr">
-        <is>
-          <t>Airbag quality/stain</t>
-        </is>
-      </c>
-      <c r="Q27" s="107" t="inlineStr">
-        <is>
-          <t>Midsole/Outsole to upper bond gap</t>
-        </is>
-      </c>
+      <c r="P27" s="125" t="inlineStr">
+        <is>
+          <t>Bottom Cosmetic</t>
+        </is>
+      </c>
+      <c r="Q27" s="230" t="n"/>
       <c r="R27" s="80" t="n"/>
       <c r="S27" s="80" t="n"/>
       <c r="T27" s="80" t="n"/>
@@ -4249,14 +4328,14 @@
       </c>
       <c r="D28" s="89" t="inlineStr">
         <is>
-          <t>NIKE INITIATOR (MS/WS)</t>
+          <t>NIKE AIR MAX EXCEE (MS/WS)</t>
         </is>
       </c>
       <c r="E28" s="90" t="n">
-        <v>187587</v>
+        <v>175514</v>
       </c>
       <c r="F28" s="90" t="n">
-        <v>5790</v>
+        <v>5267</v>
       </c>
       <c r="G28" s="109">
         <f>F28/E28</f>
@@ -4272,20 +4351,20 @@
       </c>
       <c r="L28" s="89" t="inlineStr">
         <is>
-          <t>NIKE INITIATOR (MS/WS)</t>
+          <t>NIKE AIR MAX EXCEE (MS/WS)</t>
         </is>
       </c>
       <c r="M28" s="123" t="n">
-        <v>0.139047</v>
+        <v>0.177203</v>
       </c>
       <c r="N28" s="123" t="n">
-        <v>0.09327100000000001</v>
+        <v>0.104737</v>
       </c>
       <c r="O28" s="123" t="n">
-        <v>0.115815</v>
-      </c>
-      <c r="P28" s="123" t="n"/>
-      <c r="Q28" s="124" t="n"/>
+        <v>0.143612</v>
+      </c>
+      <c r="P28" s="124" t="n"/>
+      <c r="Q28" s="233" t="n"/>
       <c r="R28" s="80" t="n"/>
       <c r="S28" s="80" t="n"/>
       <c r="T28" s="80" t="n"/>
@@ -4298,14 +4377,14 @@
       <c r="C29" s="113" t="n"/>
       <c r="D29" s="89" t="inlineStr">
         <is>
-          <t>NIKE RUN DEFY (MS/WS)</t>
+          <t>NIKE INITIATOR (MS/WS)</t>
         </is>
       </c>
       <c r="E29" s="90" t="n">
-        <v>187587</v>
+        <v>175514</v>
       </c>
       <c r="F29" s="90" t="n">
-        <v>3939</v>
+        <v>3025</v>
       </c>
       <c r="G29" s="109">
         <f>F29/E29</f>
@@ -4317,20 +4396,20 @@
       <c r="K29" s="113" t="n"/>
       <c r="L29" s="89" t="inlineStr">
         <is>
-          <t>NIKE RUN DEFY (MS/WS)</t>
+          <t>NIKE INITIATOR (MS/WS)</t>
         </is>
       </c>
       <c r="M29" s="96" t="n">
-        <v>0.14329</v>
+        <v>0.134142</v>
       </c>
       <c r="N29" s="96" t="n">
-        <v>0.117513</v>
+        <v>0.11512</v>
       </c>
       <c r="O29" s="96" t="n">
-        <v>0.112964</v>
-      </c>
-      <c r="P29" s="96" t="n"/>
-      <c r="Q29" s="97" t="n"/>
+        <v>0.09478499999999999</v>
+      </c>
+      <c r="P29" s="97" t="n"/>
+      <c r="Q29" s="231" t="n"/>
       <c r="R29" s="83" t="n"/>
       <c r="S29" s="83" t="n"/>
       <c r="T29" s="83" t="n"/>
@@ -4344,14 +4423,14 @@
       <c r="C30" s="113" t="n"/>
       <c r="D30" s="89" t="inlineStr">
         <is>
-          <t>NIKE AIR MAX EXCEE (MS/WS)</t>
+          <t>NIKE AIR MAX SC (MS/WS)</t>
         </is>
       </c>
       <c r="E30" s="90" t="n">
-        <v>187587</v>
+        <v>175514</v>
       </c>
       <c r="F30" s="90" t="n">
-        <v>3616</v>
+        <v>2409</v>
       </c>
       <c r="G30" s="109">
         <f>F30/E30</f>
@@ -4363,20 +4442,20 @@
       <c r="K30" s="113" t="n"/>
       <c r="L30" s="89" t="inlineStr">
         <is>
-          <t>NIKE AIR MAX EXCEE (MS/WS)</t>
+          <t>NIKE AIR MAX SC (MS/WS)</t>
         </is>
       </c>
       <c r="M30" s="96" t="n">
-        <v>0.185542</v>
+        <v>0.150311</v>
       </c>
       <c r="N30" s="96" t="n">
-        <v>0.138813</v>
+        <v>0.118012</v>
       </c>
       <c r="O30" s="96" t="n">
-        <v>0.121495</v>
-      </c>
-      <c r="P30" s="96" t="n"/>
-      <c r="Q30" s="97" t="n"/>
+        <v>0.143685</v>
+      </c>
+      <c r="P30" s="97" t="n"/>
+      <c r="Q30" s="231" t="n"/>
       <c r="R30" s="83" t="n"/>
       <c r="S30" s="83" t="n"/>
       <c r="T30" s="83" t="n"/>
@@ -4390,14 +4469,14 @@
       <c r="C31" s="113" t="n"/>
       <c r="D31" s="89" t="inlineStr">
         <is>
-          <t>NIKE UPLIFT SC (MS/WS)</t>
+          <t>NIKE AIR WINFLO 12 (MS/WS)</t>
         </is>
       </c>
       <c r="E31" s="90" t="n">
-        <v>187587</v>
+        <v>175514</v>
       </c>
       <c r="F31" s="90" t="n">
-        <v>1690</v>
+        <v>2189</v>
       </c>
       <c r="G31" s="109">
         <f>F31/E31</f>
@@ -4409,20 +4488,20 @@
       <c r="K31" s="113" t="n"/>
       <c r="L31" s="89" t="inlineStr">
         <is>
-          <t>NIKE UPLIFT SC (MS/WS)</t>
+          <t>NIKE AIR WINFLO 12 (MS/WS)</t>
         </is>
       </c>
       <c r="M31" s="96" t="n">
-        <v>0.157343</v>
-      </c>
-      <c r="N31" s="96" t="n"/>
-      <c r="O31" s="96" t="n">
-        <v>0.096737</v>
-      </c>
-      <c r="P31" s="96" t="n"/>
-      <c r="Q31" s="97" t="n">
-        <v>0.088578</v>
-      </c>
+        <v>0.153706</v>
+      </c>
+      <c r="N31" s="96" t="n">
+        <v>0.114598</v>
+      </c>
+      <c r="O31" s="96" t="n"/>
+      <c r="P31" s="97" t="n">
+        <v>0.109141</v>
+      </c>
+      <c r="Q31" s="231" t="n"/>
       <c r="R31" s="83" t="n"/>
       <c r="S31" s="83" t="n"/>
       <c r="T31" s="83" t="n"/>
@@ -4436,14 +4515,14 @@
       <c r="C32" s="115" t="n"/>
       <c r="D32" s="116" t="inlineStr">
         <is>
-          <t>NIKE AIR MAX SC (MS/WS)</t>
+          <t>NIKE UPLIFT SC (MS/WS)</t>
         </is>
       </c>
       <c r="E32" s="117" t="n">
-        <v>187587</v>
+        <v>175514</v>
       </c>
       <c r="F32" s="117" t="n">
-        <v>1480</v>
+        <v>2139</v>
       </c>
       <c r="G32" s="118">
         <f>F32/E32</f>
@@ -4455,20 +4534,20 @@
       <c r="K32" s="115" t="n"/>
       <c r="L32" s="116" t="inlineStr">
         <is>
-          <t>NIKE AIR MAX SC (MS/WS)</t>
+          <t>NIKE UPLIFT SC (MS/WS)</t>
         </is>
       </c>
       <c r="M32" s="119" t="n">
-        <v>0.120352</v>
+        <v>0.135455</v>
       </c>
       <c r="N32" s="119" t="n">
-        <v>0.121028</v>
-      </c>
-      <c r="O32" s="119" t="n"/>
-      <c r="P32" s="119" t="n">
-        <v>0.114943</v>
-      </c>
-      <c r="Q32" s="120" t="n"/>
+        <v>0.116818</v>
+      </c>
+      <c r="O32" s="119" t="n">
+        <v>0.096818</v>
+      </c>
+      <c r="P32" s="120" t="n"/>
+      <c r="Q32" s="231" t="n"/>
       <c r="R32" s="83" t="n"/>
       <c r="S32" s="83" t="n"/>
       <c r="T32" s="83" t="n"/>
@@ -4519,14 +4598,14 @@
       </c>
       <c r="M33" s="122" t="inlineStr">
         <is>
+          <t>Over cement</t>
+        </is>
+      </c>
+      <c r="N33" s="122" t="inlineStr">
+        <is>
           <t>Cleanness</t>
         </is>
       </c>
-      <c r="N33" s="122" t="inlineStr">
-        <is>
-          <t>Over cement</t>
-        </is>
-      </c>
       <c r="O33" s="122" t="inlineStr">
         <is>
           <t>Thread end</t>
@@ -4534,13 +4613,13 @@
       </c>
       <c r="P33" s="125" t="inlineStr">
         <is>
-          <t>Sole attachment</t>
+          <t>Bottom Cosmetic</t>
         </is>
       </c>
       <c r="Q33" s="232" t="n"/>
-      <c r="R33" s="83" t="n"/>
-      <c r="S33" s="83" t="n"/>
-      <c r="T33" s="83" t="n"/>
+      <c r="R33" s="232" t="n"/>
+      <c r="S33" s="232" t="n"/>
+      <c r="T33" s="232" t="n"/>
       <c r="U33" s="246" t="n"/>
       <c r="V33" s="80" t="n"/>
       <c r="W33" s="24" t="n"/>
@@ -4559,10 +4638,10 @@
         </is>
       </c>
       <c r="E34" s="90" t="n">
-        <v>91617</v>
+        <v>97919</v>
       </c>
       <c r="F34" s="90" t="n">
-        <v>2911</v>
+        <v>5332</v>
       </c>
       <c r="G34" s="109">
         <f>F34/E34</f>
@@ -4582,19 +4661,19 @@
         </is>
       </c>
       <c r="M34" s="96" t="n">
-        <v>0.107877</v>
+        <v>0.167945</v>
       </c>
       <c r="N34" s="96" t="n">
-        <v>0.162329</v>
+        <v>0.150365</v>
       </c>
       <c r="O34" s="96" t="n">
-        <v>0.114726</v>
+        <v>0.100991</v>
       </c>
       <c r="P34" s="124" t="n"/>
       <c r="Q34" s="233" t="n"/>
-      <c r="R34" s="80" t="n"/>
-      <c r="S34" s="80" t="n"/>
-      <c r="T34" s="80" t="n"/>
+      <c r="R34" s="242" t="n"/>
+      <c r="S34" s="242" t="n"/>
+      <c r="T34" s="242" t="n"/>
       <c r="U34" s="80" t="n"/>
       <c r="V34" s="245" t="n"/>
     </row>
@@ -4608,10 +4687,10 @@
         </is>
       </c>
       <c r="E35" s="90" t="n">
-        <v>91617</v>
+        <v>97919</v>
       </c>
       <c r="F35" s="90" t="n">
-        <v>1819</v>
+        <v>2347</v>
       </c>
       <c r="G35" s="109">
         <f>F35/E35</f>
@@ -4627,19 +4706,19 @@
         </is>
       </c>
       <c r="M35" s="123" t="n">
-        <v>0.166272</v>
+        <v>0.129422</v>
       </c>
       <c r="N35" s="123" t="n">
-        <v>0.135007</v>
+        <v>0.15231</v>
       </c>
       <c r="O35" s="123" t="n">
-        <v>0.092847</v>
+        <v>0.108198</v>
       </c>
       <c r="P35" s="124" t="n"/>
       <c r="Q35" s="233" t="n"/>
-      <c r="R35" s="80" t="n"/>
-      <c r="S35" s="80" t="n"/>
-      <c r="T35" s="80" t="n"/>
+      <c r="R35" s="242" t="n"/>
+      <c r="S35" s="242" t="n"/>
+      <c r="T35" s="242" t="n"/>
       <c r="U35" s="80" t="n"/>
       <c r="V35" s="245" t="n"/>
     </row>
@@ -4649,14 +4728,14 @@
       <c r="C36" s="113" t="n"/>
       <c r="D36" s="89" t="inlineStr">
         <is>
-          <t>NIKE AIR MAX SC (MS/WS)</t>
+          <t>NIKE AIR MAX MOTION 2 (MS/WS)</t>
         </is>
       </c>
       <c r="E36" s="90" t="n">
-        <v>91617</v>
+        <v>97919</v>
       </c>
       <c r="F36" s="90" t="n">
-        <v>1258</v>
+        <v>1246</v>
       </c>
       <c r="G36" s="109">
         <f>F36/E36</f>
@@ -4668,23 +4747,23 @@
       <c r="K36" s="113" t="n"/>
       <c r="L36" s="89" t="inlineStr">
         <is>
-          <t>NIKE AIR MAX SC (MS/WS)</t>
+          <t>NIKE AIR MAX MOTION 2 (MS/WS)</t>
         </is>
       </c>
       <c r="M36" s="96" t="n">
-        <v>0.198728</v>
-      </c>
-      <c r="N36" s="96" t="n">
-        <v>0.163752</v>
-      </c>
-      <c r="O36" s="96" t="n"/>
+        <v>0.151807</v>
+      </c>
+      <c r="N36" s="96" t="n"/>
+      <c r="O36" s="96" t="n">
+        <v>0.120482</v>
+      </c>
       <c r="P36" s="97" t="n">
-        <v>0.08267099999999999</v>
+        <v>0.135743</v>
       </c>
       <c r="Q36" s="231" t="n"/>
-      <c r="R36" s="83" t="n"/>
-      <c r="S36" s="83" t="n"/>
-      <c r="T36" s="83" t="n"/>
+      <c r="R36" s="231" t="n"/>
+      <c r="S36" s="231" t="n"/>
+      <c r="T36" s="231" t="n"/>
       <c r="U36" s="83" t="n"/>
       <c r="V36" s="241" t="n"/>
       <c r="W36" s="24" t="n"/>
@@ -4695,14 +4774,14 @@
       <c r="C37" s="113" t="n"/>
       <c r="D37" s="89" t="inlineStr">
         <is>
-          <t>NIKE COURT VISION LOW (MS/WS)</t>
+          <t>NIKE STAR RUNNER 5 (PS)</t>
         </is>
       </c>
       <c r="E37" s="90" t="n">
-        <v>91617</v>
+        <v>97919</v>
       </c>
       <c r="F37" s="90" t="n">
-        <v>687</v>
+        <v>648</v>
       </c>
       <c r="G37" s="109">
         <f>F37/E37</f>
@@ -4714,23 +4793,23 @@
       <c r="K37" s="113" t="n"/>
       <c r="L37" s="89" t="inlineStr">
         <is>
-          <t>NIKE COURT VISION LOW (MS/WS)</t>
+          <t>NIKE STAR RUNNER 5 (PS)</t>
         </is>
       </c>
       <c r="M37" s="96" t="n">
-        <v>0.126961</v>
+        <v>0.114206</v>
       </c>
       <c r="N37" s="96" t="n">
-        <v>0.11127</v>
+        <v>0.175487</v>
       </c>
       <c r="O37" s="96" t="n">
-        <v>0.108417</v>
+        <v>0.112813</v>
       </c>
       <c r="P37" s="97" t="n"/>
       <c r="Q37" s="231" t="n"/>
-      <c r="R37" s="83" t="n"/>
-      <c r="S37" s="83" t="n"/>
-      <c r="T37" s="83" t="n"/>
+      <c r="R37" s="231" t="n"/>
+      <c r="S37" s="231" t="n"/>
+      <c r="T37" s="231" t="n"/>
       <c r="U37" s="83" t="n"/>
       <c r="V37" s="241" t="n"/>
       <c r="W37" s="24" t="n"/>
@@ -4741,14 +4820,14 @@
       <c r="C38" s="115" t="n"/>
       <c r="D38" s="116" t="inlineStr">
         <is>
-          <t>NIKE AIR MAX MOTION 2 (MS/WS)</t>
+          <t>NIKE COURT BOROUGH LOW RECRAFT (TD)</t>
         </is>
       </c>
       <c r="E38" s="117" t="n">
-        <v>91617</v>
+        <v>97919</v>
       </c>
       <c r="F38" s="117" t="n">
-        <v>613</v>
+        <v>639</v>
       </c>
       <c r="G38" s="118">
         <f>F38/E38</f>
@@ -4760,23 +4839,23 @@
       <c r="K38" s="115" t="n"/>
       <c r="L38" s="116" t="inlineStr">
         <is>
-          <t>NIKE AIR MAX MOTION 2 (MS/WS)</t>
+          <t>NIKE COURT BOROUGH LOW RECRAFT (TD)</t>
         </is>
       </c>
       <c r="M38" s="119" t="n">
-        <v>0.135179</v>
+        <v>0.342723</v>
       </c>
       <c r="N38" s="119" t="n">
-        <v>0.135179</v>
+        <v>0.258216</v>
       </c>
       <c r="O38" s="119" t="n">
-        <v>0.153094</v>
+        <v>0.097027</v>
       </c>
       <c r="P38" s="120" t="n"/>
       <c r="Q38" s="231" t="n"/>
-      <c r="R38" s="83" t="n"/>
-      <c r="S38" s="83" t="n"/>
-      <c r="T38" s="83" t="n"/>
+      <c r="R38" s="231" t="n"/>
+      <c r="S38" s="231" t="n"/>
+      <c r="T38" s="231" t="n"/>
       <c r="U38" s="83" t="n"/>
       <c r="V38" s="241" t="n"/>
       <c r="W38" s="24" t="n"/>
@@ -4824,32 +4903,32 @@
       </c>
       <c r="M39" s="122" t="inlineStr">
         <is>
+          <t>Over cement</t>
+        </is>
+      </c>
+      <c r="N39" s="122" t="inlineStr">
+        <is>
           <t>Cleanness</t>
         </is>
       </c>
-      <c r="N39" s="122" t="inlineStr">
-        <is>
-          <t>Over cement</t>
-        </is>
-      </c>
       <c r="O39" s="122" t="inlineStr">
         <is>
+          <t>Midsole/Outsole to upper bond gap</t>
+        </is>
+      </c>
+      <c r="P39" s="122" t="inlineStr">
+        <is>
           <t>Thread end</t>
         </is>
       </c>
-      <c r="P39" s="122" t="inlineStr">
+      <c r="Q39" s="122" t="inlineStr">
         <is>
           <t>Toe off center</t>
         </is>
       </c>
-      <c r="Q39" s="122" t="inlineStr">
-        <is>
-          <t>Heel/Tip height inconsistent</t>
-        </is>
-      </c>
       <c r="R39" s="125" t="inlineStr">
         <is>
-          <t>Rocking</t>
+          <t>Over buffing</t>
         </is>
       </c>
       <c r="S39" s="83" t="n"/>
@@ -4872,10 +4951,10 @@
         </is>
       </c>
       <c r="E40" s="90" t="n">
-        <v>93287</v>
+        <v>79079</v>
       </c>
       <c r="F40" s="90" t="n">
-        <v>928</v>
+        <v>830</v>
       </c>
       <c r="G40" s="109">
         <f>F40/E40</f>
@@ -4895,16 +4974,16 @@
         </is>
       </c>
       <c r="M40" s="96" t="n">
-        <v>0.145022</v>
+        <v>0.160398</v>
       </c>
       <c r="N40" s="96" t="n">
-        <v>0.1829</v>
-      </c>
-      <c r="O40" s="96" t="n">
-        <v>0.102814</v>
-      </c>
+        <v>0.141593</v>
+      </c>
+      <c r="O40" s="96" t="n"/>
       <c r="P40" s="96" t="n"/>
-      <c r="Q40" s="96" t="n"/>
+      <c r="Q40" s="96" t="n">
+        <v>0.105088</v>
+      </c>
       <c r="R40" s="97" t="n"/>
       <c r="S40" s="83" t="n"/>
       <c r="T40" s="83" t="n"/>
@@ -4918,14 +4997,14 @@
       <c r="C41" s="113" t="n"/>
       <c r="D41" s="89" t="inlineStr">
         <is>
-          <t>AIR JORDAN 1 MID SE (GS)</t>
+          <t>NIKE INITIATOR (MS/WS)</t>
         </is>
       </c>
       <c r="E41" s="90" t="n">
-        <v>93287</v>
+        <v>79079</v>
       </c>
       <c r="F41" s="90" t="n">
-        <v>586</v>
+        <v>664</v>
       </c>
       <c r="G41" s="109">
         <f>F41/E41</f>
@@ -4937,20 +5016,20 @@
       <c r="K41" s="113" t="n"/>
       <c r="L41" s="89" t="inlineStr">
         <is>
-          <t>AIR JORDAN 1 MID SE (GS)</t>
+          <t>NIKE INITIATOR (MS/WS)</t>
         </is>
       </c>
       <c r="M41" s="96" t="n">
-        <v>0.2496</v>
+        <v>0.09171600000000001</v>
       </c>
       <c r="N41" s="96" t="n">
-        <v>0.1136</v>
+        <v>0.115385</v>
       </c>
       <c r="O41" s="96" t="n"/>
-      <c r="P41" s="123" t="n"/>
-      <c r="Q41" s="123" t="n">
-        <v>0.0912</v>
-      </c>
+      <c r="P41" s="123" t="n">
+        <v>0.112426</v>
+      </c>
+      <c r="Q41" s="123" t="n"/>
       <c r="R41" s="97" t="n"/>
       <c r="S41" s="80" t="n"/>
       <c r="T41" s="80" t="n"/>
@@ -4967,10 +5046,10 @@
         </is>
       </c>
       <c r="E42" s="90" t="n">
-        <v>93287</v>
+        <v>79079</v>
       </c>
       <c r="F42" s="90" t="n">
-        <v>571</v>
+        <v>387</v>
       </c>
       <c r="G42" s="109">
         <f>F42/E42</f>
@@ -4986,17 +5065,17 @@
         </is>
       </c>
       <c r="M42" s="123" t="n">
-        <v>0.144737</v>
+        <v>0.168724</v>
       </c>
       <c r="N42" s="123" t="n">
-        <v>0.184211</v>
-      </c>
-      <c r="O42" s="123" t="n">
-        <v>0.086257</v>
-      </c>
+        <v>0.13786</v>
+      </c>
+      <c r="O42" s="123" t="n"/>
       <c r="P42" s="123" t="n"/>
       <c r="Q42" s="123" t="n"/>
-      <c r="R42" s="247" t="n"/>
+      <c r="R42" s="124" t="n">
+        <v>0.096708</v>
+      </c>
       <c r="S42" s="80" t="n"/>
       <c r="T42" s="80" t="n"/>
       <c r="U42" s="80" t="n"/>
@@ -5008,14 +5087,14 @@
       <c r="C43" s="113" t="n"/>
       <c r="D43" s="89" t="inlineStr">
         <is>
-          <t>NIKE INITIATOR (MS/WS)</t>
+          <t>AIR JORDAN 1 LOW (MS/WS)</t>
         </is>
       </c>
       <c r="E43" s="90" t="n">
-        <v>93287</v>
+        <v>79079</v>
       </c>
       <c r="F43" s="90" t="n">
-        <v>563</v>
+        <v>344</v>
       </c>
       <c r="G43" s="109">
         <f>F43/E43</f>
@@ -5027,19 +5106,19 @@
       <c r="K43" s="113" t="n"/>
       <c r="L43" s="89" t="inlineStr">
         <is>
-          <t>NIKE INITIATOR (MS/WS)</t>
+          <t>AIR JORDAN 1 LOW (MS/WS)</t>
         </is>
       </c>
       <c r="M43" s="96" t="n">
-        <v>0.117229</v>
+        <v>0.205069</v>
       </c>
       <c r="N43" s="96" t="n">
-        <v>0.111901</v>
-      </c>
-      <c r="O43" s="96" t="n"/>
-      <c r="P43" s="96" t="n">
-        <v>0.094139</v>
-      </c>
+        <v>0.170507</v>
+      </c>
+      <c r="O43" s="96" t="n">
+        <v>0.085253</v>
+      </c>
+      <c r="P43" s="96" t="n"/>
       <c r="Q43" s="96" t="n"/>
       <c r="R43" s="97" t="n"/>
       <c r="S43" s="83" t="n"/>
@@ -5054,14 +5133,14 @@
       <c r="C44" s="115" t="n"/>
       <c r="D44" s="116" t="inlineStr">
         <is>
-          <t>AIR JORDAN 1 LOW (MS/WS)</t>
+          <t>AIR JORDAN 1 LOW SE (GS)</t>
         </is>
       </c>
       <c r="E44" s="117" t="n">
-        <v>93287</v>
+        <v>79079</v>
       </c>
       <c r="F44" s="117" t="n">
-        <v>440</v>
+        <v>276</v>
       </c>
       <c r="G44" s="118">
         <f>F44/E44</f>
@@ -5073,21 +5152,21 @@
       <c r="K44" s="115" t="n"/>
       <c r="L44" s="116" t="inlineStr">
         <is>
-          <t>AIR JORDAN 1 LOW (MS/WS)</t>
+          <t>AIR JORDAN 1 LOW SE (GS)</t>
         </is>
       </c>
       <c r="M44" s="119" t="n">
-        <v>0.153565</v>
+        <v>0.185759</v>
       </c>
       <c r="N44" s="119" t="n">
-        <v>0.159049</v>
-      </c>
-      <c r="O44" s="119" t="n"/>
+        <v>0.195046</v>
+      </c>
+      <c r="O44" s="119" t="n">
+        <v>0.117647</v>
+      </c>
       <c r="P44" s="119" t="n"/>
       <c r="Q44" s="119" t="n"/>
-      <c r="R44" s="120" t="n">
-        <v>0.084095</v>
-      </c>
+      <c r="R44" s="120" t="n"/>
       <c r="S44" s="83" t="n"/>
       <c r="T44" s="83" t="n"/>
       <c r="U44" s="83" t="n"/>
@@ -5133,7 +5212,7 @@
       <c r="J46" s="80" t="n"/>
       <c r="K46" s="248" t="inlineStr">
         <is>
-          <t>Defect Color Legend by Factory (Jun, 2026)</t>
+          <t>Defect Color Legend by Factory (Sep, 2026)</t>
         </is>
       </c>
       <c r="L46" s="81" t="n"/>
@@ -5262,10 +5341,10 @@
         </is>
       </c>
       <c r="M50" s="80" t="n"/>
-      <c r="N50" s="141" t="n"/>
+      <c r="N50" s="139" t="n"/>
       <c r="O50" s="135" t="inlineStr">
         <is>
-          <t>Thread end</t>
+          <t>Over cement</t>
         </is>
       </c>
       <c r="P50" s="127" t="n"/>
@@ -5289,17 +5368,17 @@
       <c r="H51" s="80" t="n"/>
       <c r="I51" s="80" t="n"/>
       <c r="J51" s="80" t="n"/>
-      <c r="K51" s="250" t="n"/>
+      <c r="K51" s="252" t="n"/>
       <c r="L51" s="135" t="inlineStr">
         <is>
-          <t>Rocking</t>
+          <t>Components inconsistent</t>
         </is>
       </c>
       <c r="M51" s="80" t="n"/>
-      <c r="N51" s="139" t="n"/>
+      <c r="N51" s="141" t="n"/>
       <c r="O51" s="135" t="inlineStr">
         <is>
-          <t>Over cement</t>
+          <t>Thread end</t>
         </is>
       </c>
       <c r="P51" s="127" t="n"/>
@@ -5323,17 +5402,17 @@
       <c r="H52" s="80" t="n"/>
       <c r="I52" s="80" t="n"/>
       <c r="J52" s="80" t="n"/>
-      <c r="K52" s="141" t="n"/>
+      <c r="K52" s="256" t="n"/>
       <c r="L52" s="135" t="inlineStr">
         <is>
-          <t>Thread end</t>
+          <t>Heel/Tip height inconsistent</t>
         </is>
       </c>
       <c r="M52" s="80" t="n"/>
-      <c r="N52" s="251" t="n"/>
+      <c r="N52" s="257" t="n"/>
       <c r="O52" s="135" t="inlineStr">
         <is>
-          <t>Airbag quality/stain</t>
+          <t>Bottom Cosmetic</t>
         </is>
       </c>
       <c r="P52" s="127" t="n"/>
@@ -5357,20 +5436,16 @@
       <c r="H53" s="80" t="n"/>
       <c r="I53" s="80" t="n"/>
       <c r="J53" s="80" t="n"/>
-      <c r="K53" s="252" t="n"/>
+      <c r="K53" s="267" t="n"/>
       <c r="L53" s="135" t="inlineStr">
         <is>
-          <t>Components inconsistent</t>
+          <t>Wrinkle bottom</t>
         </is>
       </c>
       <c r="M53" s="80" t="n"/>
-      <c r="N53" s="253" t="n"/>
-      <c r="O53" s="135" t="inlineStr">
-        <is>
-          <t>Midsole/Outsole to upper bond gap</t>
-        </is>
-      </c>
-      <c r="P53" s="127" t="n"/>
+      <c r="N53" s="80" t="n"/>
+      <c r="O53" s="245" t="n"/>
+      <c r="P53" s="80" t="n"/>
       <c r="Q53" s="80" t="n"/>
       <c r="R53" s="80" t="n"/>
       <c r="S53" s="80" t="n"/>
@@ -5391,10 +5466,10 @@
       <c r="H54" s="80" t="n"/>
       <c r="I54" s="80" t="n"/>
       <c r="J54" s="80" t="n"/>
-      <c r="K54" s="253" t="n"/>
+      <c r="K54" s="268" t="n"/>
       <c r="L54" s="135" t="inlineStr">
         <is>
-          <t>Midsole/Outsole to upper bond gap</t>
+          <t>Over buffing</t>
         </is>
       </c>
       <c r="M54" s="80" t="n"/>
@@ -5422,7 +5497,7 @@
       <c r="I55" s="80" t="n"/>
       <c r="J55" s="80" t="n"/>
       <c r="K55" s="80" t="n"/>
-      <c r="L55" s="80" t="n"/>
+      <c r="L55" s="245" t="n"/>
       <c r="M55" s="80" t="n"/>
       <c r="N55" s="80" t="n"/>
       <c r="O55" s="80" t="n"/>
@@ -5481,17 +5556,17 @@
       <c r="H57" s="80" t="n"/>
       <c r="I57" s="80" t="n"/>
       <c r="J57" s="80" t="n"/>
-      <c r="K57" s="134" t="n"/>
+      <c r="K57" s="139" t="n"/>
       <c r="L57" s="135" t="inlineStr">
         <is>
-          <t>Cleanness</t>
+          <t>Over cement</t>
         </is>
       </c>
       <c r="M57" s="80" t="n"/>
-      <c r="N57" s="134" t="n"/>
+      <c r="N57" s="139" t="n"/>
       <c r="O57" s="135" t="inlineStr">
         <is>
-          <t>Cleanness</t>
+          <t>Over cement</t>
         </is>
       </c>
       <c r="P57" s="127" t="n"/>
@@ -5515,17 +5590,17 @@
       <c r="H58" s="80" t="n"/>
       <c r="I58" s="80" t="n"/>
       <c r="J58" s="80" t="n"/>
-      <c r="K58" s="139" t="n"/>
+      <c r="K58" s="134" t="n"/>
       <c r="L58" s="135" t="inlineStr">
         <is>
-          <t>Over cement</t>
+          <t>Cleanness</t>
         </is>
       </c>
       <c r="M58" s="80" t="n"/>
-      <c r="N58" s="139" t="n"/>
+      <c r="N58" s="134" t="n"/>
       <c r="O58" s="135" t="inlineStr">
         <is>
-          <t>Over cement</t>
+          <t>Cleanness</t>
         </is>
       </c>
       <c r="P58" s="127" t="n"/>
@@ -5556,10 +5631,10 @@
         </is>
       </c>
       <c r="M59" s="80" t="n"/>
-      <c r="N59" s="141" t="n"/>
+      <c r="N59" s="253" t="n"/>
       <c r="O59" s="135" t="inlineStr">
         <is>
-          <t>Thread end</t>
+          <t>Midsole/Outsole to upper bond gap</t>
         </is>
       </c>
       <c r="P59" s="127" t="n"/>
@@ -5583,17 +5658,17 @@
       <c r="H60" s="80" t="n"/>
       <c r="I60" s="80" t="n"/>
       <c r="J60" s="80" t="n"/>
-      <c r="K60" s="254" t="n"/>
+      <c r="K60" s="257" t="n"/>
       <c r="L60" s="135" t="inlineStr">
         <is>
-          <t>Sole attachment</t>
+          <t>Bottom Cosmetic</t>
         </is>
       </c>
       <c r="M60" s="80" t="n"/>
-      <c r="N60" s="255" t="n"/>
+      <c r="N60" s="141" t="n"/>
       <c r="O60" s="135" t="inlineStr">
         <is>
-          <t>Toe off center</t>
+          <t>Thread end</t>
         </is>
       </c>
       <c r="P60" s="127" t="n"/>
@@ -5618,12 +5693,12 @@
       <c r="I61" s="80" t="n"/>
       <c r="J61" s="80" t="n"/>
       <c r="K61" s="80" t="n"/>
-      <c r="L61" s="80" t="n"/>
+      <c r="L61" s="245" t="n"/>
       <c r="M61" s="80" t="n"/>
-      <c r="N61" s="256" t="n"/>
+      <c r="N61" s="255" t="n"/>
       <c r="O61" s="135" t="inlineStr">
         <is>
-          <t>Heel/Tip height inconsistent</t>
+          <t>Toe off center</t>
         </is>
       </c>
       <c r="P61" s="127" t="n"/>
@@ -5648,12 +5723,12 @@
       <c r="I62" s="80" t="n"/>
       <c r="J62" s="80" t="n"/>
       <c r="K62" s="80" t="n"/>
-      <c r="L62" s="80" t="n"/>
+      <c r="L62" s="245" t="n"/>
       <c r="M62" s="80" t="n"/>
-      <c r="N62" s="250" t="n"/>
+      <c r="N62" s="268" t="n"/>
       <c r="O62" s="135" t="inlineStr">
         <is>
-          <t>Rocking</t>
+          <t>Over buffing</t>
         </is>
       </c>
       <c r="P62" s="127" t="n"/>
@@ -5678,7 +5753,7 @@
       <c r="I63" s="80" t="n"/>
       <c r="J63" s="80" t="n"/>
       <c r="K63" s="80" t="n"/>
-      <c r="L63" s="80" t="n"/>
+      <c r="L63" s="245" t="n"/>
       <c r="M63" s="80" t="n"/>
       <c r="N63" s="80" t="n"/>
       <c r="O63" s="80" t="n"/>
@@ -5704,7 +5779,7 @@
       <c r="I64" s="80" t="n"/>
       <c r="J64" s="80" t="n"/>
       <c r="K64" s="80" t="n"/>
-      <c r="L64" s="80" t="n"/>
+      <c r="L64" s="245" t="n"/>
       <c r="M64" s="80" t="n"/>
       <c r="N64" s="80" t="n"/>
       <c r="O64" s="80" t="n"/>
@@ -5745,9 +5820,8 @@
       <c r="X65" s="80" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="23">
+  <mergeCells count="22">
     <mergeCell ref="C40:C44"/>
-    <mergeCell ref="O53:P53"/>
     <mergeCell ref="N48:P48"/>
     <mergeCell ref="O49:P49"/>
     <mergeCell ref="C28:C32"/>

</xml_diff>